<commit_message>
Add harassment rules and manuals for いいかいご
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_社内規程一式.xlsx
+++ b/output/いいかいご_社内規程一式.xlsx
@@ -26,6 +26,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事故発生時・緊急時対応マニュアル" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="身体拘束廃止に関する指針" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="苦情対応マニュアル" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ハラスメント防止規程" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="職場ハラスメント防止規定" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ハラスメント対応マニュアル" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="利用者等ハラスメント規程" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="利用者等ハラスメントマニュアル" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,7 +40,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,6 +99,11 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="20"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -129,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -206,6 +216,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10933,6 +10946,3965 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E144"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>株式会社dhpケアマネジメント　いいかいご</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1"/>
+    <row r="3" ht="24" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1"/>
+    <row r="5" ht="24" customHeight="1"/>
+    <row r="6" ht="24" customHeight="1"/>
+    <row r="7" ht="24" customHeight="1"/>
+    <row r="8" ht="24" customHeight="1"/>
+    <row r="9" ht="24" customHeight="1"/>
+    <row r="10" ht="24" customHeight="1"/>
+    <row r="11" ht="24" customHeight="1"/>
+    <row r="12" ht="24" customHeight="1"/>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>ハラスメント防止規程</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1"/>
+    <row r="15" ht="24" customHeight="1"/>
+    <row r="16" ht="24" customHeight="1"/>
+    <row r="17" ht="24" customHeight="1"/>
+    <row r="18" ht="24" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1"/>
+    <row r="21" ht="24" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1"/>
+    <row r="23" ht="24" customHeight="1"/>
+    <row r="24" ht="24" customHeight="1"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>施行　令和8年2月1日</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>第1章　総則</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>（目的）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>第1条　本規程は、株式会社dhpケアマネジメント　いいかいご（以下「会社」という。）における各種ハラスメントを防止し、発生時には迅速かつ適正に対応し、従業員が安心して働ける職場環境を確保することを目的とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="8" customHeight="1"/>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>（適用範囲）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>第2条　本規程は、会社に雇用されるすべての従業員に適用する。役員、派遣社員、アルバイト、業務委託先を含む関係者についても、会社が必要と認める範囲で適用する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="8" customHeight="1"/>
+    <row r="33" ht="8" customHeight="1">
+      <c r="A33" s="7" t="inlineStr"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+    </row>
+    <row r="34" ht="10" customHeight="1"/>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>第2章　定義</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>（ハラスメントの種類）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>第3条　本規程における「ハラスメント」とは、次に掲げる行為をいう。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>1．パワーハラスメント（パワハラ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　職場において優位な立場を背景に、業務上必要かつ相当な範囲を超えて他人の就業環境を害する行為をいう。代表例は以下のとおりとする。なお、客観的にみて、業務上必要かつ相当な範囲で行われる適正な業務指示や指導については、パワーハラスメントには該当しない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 身体的攻撃（暴行・傷害）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 精神的攻撃（侮辱・威圧的発言・過度な叱責・人格否定）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 人間関係からの切り離し（無視、隔離、仲間外し）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 過大な要求（遂行不可能な業務の押し付け）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 過小な要求（業務を与えない、能力発揮を妨げる）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 個の侵害（私生活への過度な干渉、プライバシー侵害、性的指向・性自認や病歴等の機微な個人情報の暴露）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="8" customHeight="1"/>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>2．セクシュアルハラスメント（セクハラ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　性的言動により他人に不快感や不利益を与える行為をいう。相手の性的指向又は性自認にかかわらず、同性に対する言動も該当する。代表例は以下のとおりとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 不必要な身体接触や性的な冗談・発言</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 性的な噂の流布や性的評価の強要</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 性的関係を断ったことを理由に不利益を与える行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 職場外であっても業務上の関係に基づき行われた性的言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="8" customHeight="1"/>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>3．妊娠・出産・育児・介護に関するハラスメント（マタハラ・パタハラ・ケアハラ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="48" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　妊娠・出産・育児休業・介護休業等の制度の利用に関する不利益取扱いや嫌がらせ行為をいう。なお、業務分担や安全配慮等の観点から、客観的にみて業務上の必要性に基づく言動は該当しない。例として以下がある。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 妊娠・出産・休業取得を理由とする解雇・降格・減給</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 休業取得希望に対する嫌味や阻害的言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- 育児・介護を理由とした合理性のない不利益取扱い</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="8" customHeight="1"/>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>4．その他のハラスメント</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- モラルハラスメント（人格否定、悪意のある無視）</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- SOGIハラスメント（性的指向・性自認に関する差別的言動）</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- リモートハラスメント（オンライン会議での過剰な監視・侮辱）</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="32" customHeight="1">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- カスタマーハラスメント（利用者・家族・取引先からの著しい迷惑行為。「利用者等からのハラスメント防止・対応規程」による）</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- アルコールハラスメント（飲酒の強要、不適切な酒席での言動）</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- スモークハラスメント（喫煙に関する迷惑行為）</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　- その他職場環境を不当に害する行為 等</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="8" customHeight="1"/>
+    <row r="69" ht="8" customHeight="1">
+      <c r="A69" s="7" t="inlineStr"/>
+      <c r="B69" s="8" t="n"/>
+      <c r="C69" s="8" t="n"/>
+      <c r="D69" s="8" t="n"/>
+      <c r="E69" s="8" t="n"/>
+    </row>
+    <row r="70" ht="10" customHeight="1"/>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>第3章　禁止と責務</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>（禁止行為）</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="32" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>第4条　従業員は、前条に掲げるあらゆる形態のハラスメントを行ってはならない。また、利用者・取引先等の従業員以外の者に対しても、これに類する行為を行ってはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="8" customHeight="1"/>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>（従業員の責務）</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="32" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>第5条　従業員は、健全な職場環境を維持するため、互いを尊重し、ハラスメントの未然防止に努めなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="8" customHeight="1"/>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>（管理職の責務）</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="48" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>第6条　管理職は、自らハラスメントを行わないことはもとより、部下間のハラスメントを防止し、発生時には速やかに会社へ報告しなければならない。部下がハラスメントを受けている事実を認めながら、これを黙認してはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="8" customHeight="1"/>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>（会社の責務）</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="32" customHeight="1">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>第7条　会社は、ハラスメント防止に関する方針を明示し、相談窓口を設け、教育・啓発を行い、発生時には迅速かつ適正に対応しなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="8" customHeight="1"/>
+    <row r="84" ht="8" customHeight="1">
+      <c r="A84" s="7" t="inlineStr"/>
+      <c r="B84" s="8" t="n"/>
+      <c r="C84" s="8" t="n"/>
+      <c r="D84" s="8" t="n"/>
+      <c r="E84" s="8" t="n"/>
+    </row>
+    <row r="85" ht="10" customHeight="1"/>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>第4章　相談・通報</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>（相談窓口）</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="32" customHeight="1">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>第8条　会社は、従業員が安心して相談できるよう、相談窓口を設置し、可能な限り男女各1名以上の相談担当者を置く。相談担当者は管理者（生田 友哉）及び会社が指名する者とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>2　相談は、面談、電話、電子メール、手紙、匿名通報等の方法により受け付ける。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>3　相談者のプライバシーは厳格に保護し、相談したことを理由に不利益取扱いをしてはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>4　相談への具体的な対応は「ハラスメント対応マニュアル」による。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="8" customHeight="1"/>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>（外部相談機関の活用）</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="32" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>第9条　会社は、必要に応じて弁護士、社会保険労務士、行政機関（大阪労働局 総合労働相談コーナー等）を外部相談窓口として指定することができる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="8" customHeight="1"/>
+    <row r="96" ht="8" customHeight="1">
+      <c r="A96" s="7" t="inlineStr"/>
+      <c r="B96" s="8" t="n"/>
+      <c r="C96" s="8" t="n"/>
+      <c r="D96" s="8" t="n"/>
+      <c r="E96" s="8" t="n"/>
+    </row>
+    <row r="97" ht="10" customHeight="1"/>
+    <row r="98" ht="30" customHeight="1">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>第5章　調査・是正</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>（調査）</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>第10条　会社は、相談または通報を受けた場合、速やかに事実関係を確認しなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>2　調査にあたっては、公平性を確保し、関係者に十分な意見聴取の機会を与える。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>3　調査への協力を求められた従業員は、正当な理由なくこれを拒んではならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="8" customHeight="1"/>
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>（是正措置）</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="48" customHeight="1">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>第11条　会社は、事実確認の結果、ハラスメント行為が認められた場合、加害者に対し指導、配置転換、懲戒処分等の適切な措置を講じるとともに、被害者の労働条件及び就業環境の改善、メンタルケア等の措置を講じる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="20" customHeight="1">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>2　相談者・協力者に対する二次被害を防止するため、必要な措置を講じなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>3　事実が確認できなかった場合も、職場環境の見直しと防止策の徹底を行う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="8" customHeight="1"/>
+    <row r="109" ht="8" customHeight="1">
+      <c r="A109" s="7" t="inlineStr"/>
+      <c r="B109" s="8" t="n"/>
+      <c r="C109" s="8" t="n"/>
+      <c r="D109" s="8" t="n"/>
+      <c r="E109" s="8" t="n"/>
+    </row>
+    <row r="110" ht="10" customHeight="1"/>
+    <row r="111" ht="30" customHeight="1">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>第6章　再発防止</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>（教育・研修）</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="32" customHeight="1">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>第12条　会社は、全従業員（登録ヘルパーを含む）を対象に、ハラスメント防止に関する教育・研修を入社時及び年1回以上実施する。管理職向け研修は特に重点的に実施する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="32" customHeight="1">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>2　性別役割分担意識に基づく言動や、妊娠・出産・育児・介護休業等に関する否定的な言動は、ハラスメントの原因や背景となり得ることを研修等で周知する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="8" customHeight="1"/>
+    <row r="116" ht="20" customHeight="1">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>（再発防止措置）</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="32" customHeight="1">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>第13条　会社は、ハラスメントが発生した場合、その原因を分析し、方針の再周知、研修の実施その他職場環境の改善に必要な再発防止措置を講じなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="8" customHeight="1"/>
+    <row r="119" ht="20" customHeight="1">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>（定期報告）</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="32" customHeight="1">
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t>第14条　会社は、相談・通報・対応状況について、個人情報を除いた概要を定期的に取りまとめ、代表取締役に報告し、従業員に周知する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="8" customHeight="1"/>
+    <row r="122" ht="8" customHeight="1">
+      <c r="A122" s="7" t="inlineStr"/>
+      <c r="B122" s="8" t="n"/>
+      <c r="C122" s="8" t="n"/>
+      <c r="D122" s="8" t="n"/>
+      <c r="E122" s="8" t="n"/>
+    </row>
+    <row r="123" ht="10" customHeight="1"/>
+    <row r="124" ht="30" customHeight="1">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>第7章　懲戒</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>（懲戒との関係）</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="32" customHeight="1">
+      <c r="A126" s="6" t="inlineStr">
+        <is>
+          <t>第15条　従業員が本規程に違反しハラスメント行為を行った場合は、「懲戒規程」に基づき懲戒処分の対象とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="8" customHeight="1"/>
+    <row r="128" ht="8" customHeight="1">
+      <c r="A128" s="7" t="inlineStr"/>
+      <c r="B128" s="8" t="n"/>
+      <c r="C128" s="8" t="n"/>
+      <c r="D128" s="8" t="n"/>
+      <c r="E128" s="8" t="n"/>
+    </row>
+    <row r="129" ht="10" customHeight="1"/>
+    <row r="130" ht="30" customHeight="1">
+      <c r="A130" s="4" t="inlineStr">
+        <is>
+          <t>第8章　その他</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="20" customHeight="1">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>（秘密保持義務）</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="32" customHeight="1">
+      <c r="A132" s="6" t="inlineStr">
+        <is>
+          <t>第16条　会社は、相談・調査・対応の過程で知り得た個人情報を適切に管理し、業務遂行上必要な場合を除き、第三者に開示してはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="8" customHeight="1"/>
+    <row r="134" ht="20" customHeight="1">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>（不利益取扱い禁止）</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="32" customHeight="1">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>第17条　会社は、相談者、協力者、証人となった者等に対して、不利益な取扱いをしてはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="8" customHeight="1"/>
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>（社内外への周知）</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="32" customHeight="1">
+      <c r="A138" s="6" t="inlineStr">
+        <is>
+          <t>第18条　会社は、本規程の内容を従業員に周知し、事業所内への掲示等により常時確認できる状態にしておかなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="8" customHeight="1"/>
+    <row r="140" ht="8" customHeight="1">
+      <c r="A140" s="7" t="inlineStr"/>
+      <c r="B140" s="8" t="n"/>
+      <c r="C140" s="8" t="n"/>
+      <c r="D140" s="8" t="n"/>
+      <c r="E140" s="8" t="n"/>
+    </row>
+    <row r="141" ht="10" customHeight="1"/>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>附則</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="20" customHeight="1">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>1　本規程に定めのない事項は、就業規則その他関係規程による。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>2　本規程は令和8年2月1日から施行する。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="93">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A142:E142"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A94:E94"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A87:E87"/>
+    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A128:E128"/>
+    <mergeCell ref="A137:E137"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A89:E89"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A113:E113"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="A91:E91"/>
+    <mergeCell ref="A131:E131"/>
+    <mergeCell ref="A100:E100"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A130:E130"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A138:E138"/>
+    <mergeCell ref="A132:E132"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A119:E119"/>
+    <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A120:E120"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A104:E104"/>
+    <mergeCell ref="A106:E106"/>
+    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A124:E124"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A86:E86"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A135:E135"/>
+    <mergeCell ref="A144:E144"/>
+    <mergeCell ref="A122:E122"/>
+    <mergeCell ref="A125:E125"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A134:E134"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A114:E114"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A98:E98"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A107:E107"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A88:E88"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="A99:E99"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A76:E76"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A116:E116"/>
+    <mergeCell ref="A126:E126"/>
+    <mergeCell ref="A140:E140"/>
+    <mergeCell ref="A109:E109"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A62:E62"/>
+    <mergeCell ref="A102:E102"/>
+    <mergeCell ref="A117:E117"/>
+    <mergeCell ref="A111:E111"/>
+    <mergeCell ref="A143:E143"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;9 株式会社dhpケアマネジメント　いいかいご　ハラスメント防止規程</oddHeader>
+    <oddFooter>&amp;C&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="25" min="0" max="16383" man="1"/>
+  </rowBreaks>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E84"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>株式会社dhpケアマネジメント　いいかいご</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1"/>
+    <row r="3" ht="24" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1"/>
+    <row r="5" ht="24" customHeight="1"/>
+    <row r="6" ht="24" customHeight="1"/>
+    <row r="7" ht="24" customHeight="1"/>
+    <row r="8" ht="24" customHeight="1"/>
+    <row r="9" ht="24" customHeight="1"/>
+    <row r="10" ht="24" customHeight="1"/>
+    <row r="11" ht="24" customHeight="1"/>
+    <row r="12" ht="24" customHeight="1"/>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>職場におけるハラスメントの
+防止に関する規定</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1"/>
+    <row r="15" ht="24" customHeight="1"/>
+    <row r="16" ht="24" customHeight="1"/>
+    <row r="17" ht="24" customHeight="1"/>
+    <row r="18" ht="24" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1"/>
+    <row r="21" ht="24" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1"/>
+    <row r="23" ht="24" customHeight="1"/>
+    <row r="24" ht="24" customHeight="1"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>施行　令和8年2月1日</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>（目的）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>第1条　本規定は、職場におけるパワーハラスメント、セクシュアルハラスメント及び妊娠・出産・育児休業等に関するハラスメント（以下「職場におけるハラスメント」という）を防止するために従業員が遵守するべき事項を定める。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　なお、この規定にいう従業員とは、正社員だけではなく、契約社員・登録ヘルパー等の非正規社員及び派遣労働者も含まれるものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="8" customHeight="1"/>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>（パワーハラスメント、セクシュアルハラスメント及び妊娠・出産・育児休業等に関するハラスメントの定義）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="64" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>第2条　パワーハラスメントとは、優越的な関係を背景とした言動であって、業務上必要かつ相当な範囲を超えたものにより、就業環境を害することをいう。なお、客観的にみて、業務上必要かつ相当な範囲で行われる適正な業務指示や指導については、職場におけるパワーハラスメントには該当しない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="64" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>2　セクシュアルハラスメントとは、職場における性的な言動に対する他の従業員の対応等により当該従業員の労働条件に関して不利益を与えること又は性的な言動により他の従業員の就業環境を害することをいう。また、相手の性的指向又は性自認の状況にかかわらないほか、異性に対する言動だけでなく、同性に対する言動も該当する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>3　前項の他の従業員とは直接的に性的な言動の相手方となった被害者に限らず、性的な言動により就業環境を害されたすべての従業員を含むものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="80" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>4　妊娠・出産・育児休業等に関するハラスメントとは、職場において、上司や同僚が、従業員の妊娠・出産及び育児・介護等に関する制度又は措置の利用に関する言動により従業員の就業環境を害すること並びに妊娠・出産等に関する言動により女性従業員の就業環境を害することをいう。なお、業務分担や安全配慮等の観点から、客観的にみて、業務上の必要性に基づく言動によるものについては、妊娠・出産・育児休業等に関するハラスメントには該当しない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>5　第1項、第2項及び第4項の職場とは、事業所のみならず、利用者宅その他従業員が業務を遂行するすべての場所をいい、また、就業時間内に限らず、実質的に職場の延長とみなされる就業時間外の時間を含むものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="8" customHeight="1"/>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>（禁止行為）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="64" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>第3条　すべての従業員は、他の従業員を業務遂行上の対等なパートナーとして認め、職場における健全な秩序並びに協力関係を保持する義務を負うとともに、その言動に注意を払い、職場内において次の第2項から第5項に掲げる行為をしてはならない。また、自社の従業員以外の者に対しても、これに類する行為を行ってはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>2　パワーハラスメント（第2条第1項の要件を満たした以下のような行為）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　① 殴打、足蹴りするなどの身体的攻撃</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　② 人格を否定するような言動をするなどの精神的な攻撃</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　③ 自身の意に沿わない従業員に対して、仕事を外し、長期間にわたり、別室に隔離するなどの人間関係からの切り離し</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　④ 長期間にわたり、肉体的苦痛を伴う過酷な環境下で、勤務に直接関係ない作業を命じるなどの過大な要求</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　⑤ 管理職である部下を退職させるため誰でも遂行可能な業務を行わせるなどの過小な要求</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　⑥ 他の従業員の性的指向・性自認や病歴などの機微な個人情報について本人の了解を得ずに他の従業員に暴露するなどの個の侵害</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>3　セクシュアルハラスメント（第2条第2項の要件を満たした以下のような行為）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　① 性的及び身体上の事柄に関する不必要な質問・発言</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　② わいせつ図画の閲覧、配付、掲示</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　③ うわさの流布</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　④ 不必要な身体への接触</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　⑤ 性的な言動により、他の従業員の就業意欲を低下せしめ、能力の発揮を阻害する行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　⑥ 交際・性的関係の強要</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　⑦ 性的な言動への抗議又は拒否等を行った従業員に対して、解雇、不当な人事考課、配置転換等の不利益を与える行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　⑧ その他、相手方及び他の従業員に不快感を与える性的な言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>4　妊娠・出産・育児休業等に関するハラスメント（第2条第4項の要件を満たした以下のような行為）</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　① 部下の妊娠・出産、育児・介護に関する制度や措置の利用等に関し、解雇その他不利益な取扱いを示唆する言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　② 部下又は同僚の妊娠・出産、育児・介護に関する制度や措置の利用を阻害する言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　③ 部下又は同僚が妊娠・出産、育児・介護に関する制度や措置を利用したことによる嫌がらせ等</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　④ 部下が妊娠・出産等したことにより、解雇その他の不利益な取扱いを示唆する言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　⑤ 部下又は同僚が妊娠・出産等したことに対する嫌がらせ等</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="32" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>5　部下である従業員が職場におけるハラスメントを受けている事実を認めながら、これを黙認する上司の行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="8" customHeight="1"/>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>（懲戒）</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="32" customHeight="1">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>第4条　次の各号に掲げる場合に応じ、当該各号に定める懲戒処分を行う。処分の手続は「懲戒規程」による。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>1　第3条第2項（①を除く。）、第3条第3項①から⑤及び⑧並びに第4項の行為を行った場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　懲戒規程に定めるけん責（譴責）、減給、出勤停止又は降格</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="32" customHeight="1">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>2　前号の行為が再度に及んだ場合、その情状が悪質と認められる場合、第3条第2項①又は第3条第3項⑥、⑦の行為を行った場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　懲戒規程に定める懲戒解雇</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="8" customHeight="1"/>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>（相談及び苦情への対応）</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="48" customHeight="1">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>第5条　職場におけるハラスメントに関する相談及び苦情処理の相談窓口の責任者は代表取締役とし、相談担当者は管理者（生田 友哉）とする。代表取締役は、担当者に対する対応マニュアルの作成及び対応に必要な研修を行うものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="48" customHeight="1">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>2　職場におけるハラスメントの被害者に限らず、すべての従業員は、パワーハラスメントや性的な言動、妊娠・出産・育児休業等に関する就業環境を害する言動に関する相談及び苦情を相談窓口の担当者に申し出ることができる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="48" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>3　対応マニュアルに沿い、相談窓口の担当者は相談者のプライバシーに配慮した上で、被害者、行為者から事実関係を聴取する。また、必要に応じて当事者の上司、その他の従業員から事情を聴くことができる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>4　前項の聴取を求められた従業員は、正当な理由なくこれを拒むことはできない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="32" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>5　対応マニュアルに沿い、問題解決のための措置として、第4条による懲戒の他、行為者の異動等被害者の労働条件及び就業環境を改善するために必要な措置を講じる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="32" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>6　相談及び苦情への対応に当たっては、関係者のプライバシーは保護されるとともに、相談をしたこと又は事実関係の確認に協力したこと等を理由として不利益な取扱いは行わない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="8" customHeight="1"/>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>（再発防止の義務）</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="48" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>第6条　代表取締役は、職場におけるハラスメント事案が生じた時は、周知の再徹底及び研修の実施、事案発生の原因の分析と再発防止等、会社全体の業務体制の整備等、適切な再発防止策を講じなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="8" customHeight="1"/>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>（その他）</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="64" customHeight="1">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>第7条　性別役割分担意識に基づく言動は、セクシュアルハラスメントの発生の原因や要因になり得ること、また、妊娠・出産・育児休業等に関する否定的な言動は、妊娠・出産・育児休業等に関するハラスメントの発生の原因や背景となり得ることから、このような言動を行わないよう注意すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="8" customHeight="1"/>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>附則　本規定は令和8年2月1日より実施する。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="55">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A76:E76"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A67:E67"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;9 株式会社dhpケアマネジメント　いいかいご　職場におけるハラスメントの防止に関する規定</oddHeader>
+    <oddFooter>&amp;C&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="25" min="0" max="16383" man="1"/>
+  </rowBreaks>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E111"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>株式会社dhpケアマネジメント　いいかいご</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1"/>
+    <row r="3" ht="24" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1"/>
+    <row r="5" ht="24" customHeight="1"/>
+    <row r="6" ht="24" customHeight="1"/>
+    <row r="7" ht="24" customHeight="1"/>
+    <row r="8" ht="24" customHeight="1"/>
+    <row r="9" ht="24" customHeight="1"/>
+    <row r="10" ht="24" customHeight="1"/>
+    <row r="11" ht="24" customHeight="1"/>
+    <row r="12" ht="24" customHeight="1"/>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>ハラスメント対応マニュアル</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1"/>
+    <row r="15" ht="24" customHeight="1"/>
+    <row r="16" ht="24" customHeight="1"/>
+    <row r="17" ht="24" customHeight="1"/>
+    <row r="18" ht="24" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1"/>
+    <row r="21" ht="24" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1"/>
+    <row r="23" ht="24" customHeight="1"/>
+    <row r="24" ht="24" customHeight="1"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>施行　令和8年2月1日</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Ⅰ．相談・苦情への対応のために</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>ハラスメントに関する相談・苦情を受けた場合、本マニュアルに基づき対応することとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>なお、職場におけるハラスメントが現実に生じている場合だけでなく、その発生のおそれがある場合や、職場におけるハラスメントに該当するか否か微妙な場合であっても、相談・苦情に対応するものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="10" customHeight="1"/>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>［1］相談窓口の設置</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>1．相談方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　原則面談によるものとするが、電話、手紙、電子メールも可とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2．相談窓口担当者</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　担当者は、可能な限り男女各1名以上とし、相談者が相談しやすい構成とする。担当者に対しては、定期的な研修を行い、資質の向上を図ることとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　相談担当者（ 管理者　生田 友哉 ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>3．適切な対応のために</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　相談、苦情への対応は、別添フローチャートによる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="8" customHeight="1"/>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>［2］相談窓口担当者の心得</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　1．初めに相談を受けた者の対応によっては問題が大きくなりかねないことから、初期対応は非常に重要であり、適切、迅速に対応すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　2．相談者やその相談内容に関係する者のプライバシーや名誉などを尊重し、知り得た事実の秘密を厳守すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3．相談は公正真摯な態度で、丁寧に聞くこと。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　4．相談者が面接による相談を望まない場合は、手紙、電話等の方法によることも教示すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　5．相談者の直面する問題の把握が大切であり、そのために不安感を取り除く等の配慮をしながら、解決策を考えること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　6．解決のための行動を起こす場合には、その都度事前に相談者にその旨を伝え、意向を確認しながら行うこと。</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　7．解決に時間を要するおそれのある場合は、相談者にその旨と所要日数の見込みを伝え、その後も、相談者に不安を与えないため、進捗状況を知らせながら進めること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　8．相談の対象は、ハラスメントにあたるかどうか厳密に判断するのではなく、放置しておけばハラスメントになってしまうものもあるので幅広く対象とすること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="8" customHeight="1"/>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>［3］相談・苦情の受け方</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>1．相談内容の聴取</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>相談の中で次の事項について確認する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（1）相談者と行為者の関係（上司・部下・同僚・利用者宅での同行者等）</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（2）問題とされる言動がいつ、どこで、どのように行われたか</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（3）行為者の言動に対し相談者はどのように感じ、どのような対応をとったか、また、それに対する行為者の反応</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（4）行為者の言動について、以前にこのような言動を行ったなど聞いたことがあるか、また、他の人に対しても同様な言動がなされているか</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（5）上司等に対する相談は行ったか</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（6）現在の相談者と行為者との状況はどうか</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="8" customHeight="1"/>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>2．相談に当たっての留意点</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="32" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（1）相談者からの話は、本人の了解を得た上で、相談者と担当者の認識のずれをなくすためにきちんと記録しておくこと。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="32" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（2）相談者の求める援助が、加害者に言動を止めるよう求めているか、不利益の回復なのか、謝罪を要求するか、職場全体としての対処を望むのか等、的確に把握すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（3）相談者の様子をよく観察して、対応に時間的な余裕があるかどうかを見極めること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="32" customHeight="1">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（4）相談者の意向を踏まえ、解決方法やこれからの手順を説明するとともに、当面の対処の仕方についてアドバイスすること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="8" customHeight="1"/>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>3．相談対応後の対処</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="32" customHeight="1">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　事実関係を調査する苦情処理担当との連携を密にすること。担当以外の者にこの件で接触しようとする場合は、必ず相談者に事前に同意を得ること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="10" customHeight="1"/>
+    <row r="68" ht="26" customHeight="1">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>Ⅱ．事後の迅速・適切な対応のために</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>［1］苦情処理担当</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="32" customHeight="1">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>職場でハラスメントが発生した場合の対応として、相談窓口のほか苦情処理担当を設けることとする。苦情処理担当は、公正かつ客観的な立場で対処する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>苦情処理担当は、代表取締役とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="8" customHeight="1"/>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>［2］迅速な事実確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　1．苦情処理担当は、事実の確認のため迅速に事情聴取を行うこと。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　2．把握した事実関係、対応状況等についての記録を作成し、保管しておくこと。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3．事実確認の過程であっても、必要に応じて適切な応急措置を講ずること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　4．被害者からの事実確認について</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="32" customHeight="1">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　　苦情処理担当が、相談記録に基づいて、事実関係を改めて被害者に確認すること。ハラスメントの内容が公になり、職場に居づらくなるようなことがないよう、担当は十分配慮すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　5．加害者とされた従業員からの事情聴取について</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="48" customHeight="1">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　　被害者の相談内容を説明した上で、事実関係についての事情聴取を行うと同時に、十分な弁明の機会を与えること。なお、加害者とされる者のプライバシーが十分守られるよう、細心の注意を払い事情聴取すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　6．当事者双方の言い分が食い違っている場合等には、職場の同僚等からの事実確認も行うこと。</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="32" customHeight="1">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　7．事実確認をした者が管理者である場合は、管理者は、代表取締役に事実確認した内容を報告すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="8" customHeight="1"/>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="16" t="inlineStr">
+        <is>
+          <t>［3］事実に基づく適正な対処</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="32" customHeight="1">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　1．相談したこと、又は事実関係の確認に協力したこと等を理由として不利益な取扱いは行わない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　2．事案に対しては問題の深刻度や緊急性に応じた措置を講ずること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="32" customHeight="1">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　（1）加害者に対する注意（問題となっている言動の中止、注意喚起など）や、加害者の監督者に対して状況の観察等を要請する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="32" customHeight="1">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　（2）加害者の担当利用者や勤務シフトを変更する等、当事者を引き離すよう人事上の配慮を行う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　（3）当事者間の関係改善について援助を行う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　（4）被害者に労働条件、就業環境上の不利益が存在している場合には、それを回復する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　（5）被害者の精神的ショックが大きい場合には、メンタルケアに配慮する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　（6）就業規則及び懲戒規程に基づき、加害者に一定の制裁を行う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3．事案に関し具体的に講じられた措置について、当事者に説明すること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　4．会社全体で再発防止策を講ずること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="8" customHeight="1"/>
+    <row r="96" ht="28" customHeight="1">
+      <c r="A96" s="24" t="inlineStr">
+        <is>
+          <t>相談苦情への対応の流れ（フローチャート）</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="10" customHeight="1"/>
+    <row r="98" ht="28" customHeight="1">
+      <c r="B98" s="17" t="inlineStr">
+        <is>
+          <t>相談・苦情</t>
+        </is>
+      </c>
+      <c r="C98" s="22" t="n"/>
+      <c r="D98" s="22" t="n"/>
+    </row>
+    <row r="99" ht="16" customHeight="1">
+      <c r="C99" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="46" customHeight="1">
+      <c r="B100" s="17" t="inlineStr">
+        <is>
+          <t>相談・苦情窓口
+（相談担当者：管理者 生田 友哉／苦情処理担当：代表取締役）</t>
+        </is>
+      </c>
+      <c r="C100" s="22" t="n"/>
+      <c r="D100" s="22" t="n"/>
+    </row>
+    <row r="101" ht="16" customHeight="1">
+      <c r="C101" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="28" customHeight="1">
+      <c r="B102" s="17" t="inlineStr">
+        <is>
+          <t>事実関係の確認</t>
+        </is>
+      </c>
+      <c r="C102" s="22" t="n"/>
+      <c r="D102" s="22" t="n"/>
+    </row>
+    <row r="103" ht="16" customHeight="1">
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="40" customHeight="1">
+      <c r="B104" s="17" t="inlineStr">
+        <is>
+          <t>相談者からの
+ヒヤリング</t>
+        </is>
+      </c>
+      <c r="C104" s="17" t="inlineStr">
+        <is>
+          <t>加害者とされた者
+からのヒヤリング</t>
+        </is>
+      </c>
+      <c r="D104" s="17" t="inlineStr">
+        <is>
+          <t>同僚など第三者
+からのヒヤリング</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="16" customHeight="1">
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="30" customHeight="1">
+      <c r="B106" s="17" t="inlineStr">
+        <is>
+          <t>事実が確認された</t>
+        </is>
+      </c>
+      <c r="D106" s="17" t="inlineStr">
+        <is>
+          <t>事実が確認されない</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="70" customHeight="1">
+      <c r="B107" s="17" t="inlineStr">
+        <is>
+          <t>会社の対応を検討</t>
+        </is>
+      </c>
+      <c r="D107" s="17" t="inlineStr">
+        <is>
+          <t>職場環境の見直しと
+防止策の徹底
+相談者への説明
+当事者間の関係改善の援助</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="16" customHeight="1">
+      <c r="B108" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="82" customHeight="1">
+      <c r="B109" s="17" t="inlineStr">
+        <is>
+          <t>雇用管理上の措置（担当変更、不利益回復やメンタルケア、当事者間の関係改善の援助等）
+相談者への説明
+就業規則・懲戒規程に基づく加害者への制裁（けん責、出勤停止、懲戒解雇等）
+職場環境の見直しと再発防止策の徹底</t>
+        </is>
+      </c>
+      <c r="C109" s="22" t="n"/>
+      <c r="D109" s="22" t="n"/>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>＜附則＞</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>本マニュアルは、令和8年2月1日から施行する。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="71">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="B98:D98"/>
+    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A94:E94"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A88:E88"/>
+    <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A87:E87"/>
+    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A89:E89"/>
+    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A80:E80"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A86:E86"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A76:E76"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="B100:D100"/>
+    <mergeCell ref="B109:D109"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A91:E91"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A62:E62"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="B102:D102"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A111:E111"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A92:E92"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;9 株式会社dhpケアマネジメント　いいかいご　ハラスメント対応マニュアル</oddHeader>
+    <oddFooter>&amp;C&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="25" min="0" max="16383" man="1"/>
+    <brk id="95" min="0" max="16383" man="1"/>
+  </rowBreaks>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E169"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>株式会社dhpケアマネジメント　いいかいご</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1"/>
+    <row r="3" ht="24" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1"/>
+    <row r="5" ht="24" customHeight="1"/>
+    <row r="6" ht="24" customHeight="1"/>
+    <row r="7" ht="24" customHeight="1"/>
+    <row r="8" ht="24" customHeight="1"/>
+    <row r="9" ht="24" customHeight="1"/>
+    <row r="10" ht="24" customHeight="1"/>
+    <row r="11" ht="24" customHeight="1"/>
+    <row r="12" ht="24" customHeight="1"/>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>利用者等からのハラスメント
+防止・対応規程</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1"/>
+    <row r="15" ht="24" customHeight="1"/>
+    <row r="16" ht="24" customHeight="1"/>
+    <row r="17" ht="24" customHeight="1"/>
+    <row r="18" ht="24" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1"/>
+    <row r="21" ht="24" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1"/>
+    <row r="23" ht="24" customHeight="1"/>
+    <row r="24" ht="24" customHeight="1"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>施行　令和8年2月1日</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>第1章　総則</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>（目的）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="80" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>第1条　本規程は、株式会社dhpケアマネジメント　いいかいご（以下「会社」という）の従業員が、利用者またはその家族その他の関係者（以下「利用者等」という）からのハラスメント行為により、心身の安全や就労環境を害されることを防止し、安心して職務に従事できる体制を確保することを目的とする。あわせて、労働契約法、労働安全衛生法その他関係法令の趣旨に則り、会社の安全配慮義務を明確にする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="8" customHeight="1"/>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>（適用範囲）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>第2条　本規程は、会社に勤務する全従業員（正社員、契約社員、嘱託社員、パートタイマー、アルバイト、登録ヘルパー、派遣社員を含む）に適用する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>2　本規程は、利用者等によるハラスメントを対象とし、従業員間のハラスメントについては「ハラスメント防止規程」及び「職場におけるハラスメントの防止に関する規定」を適用する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="8" customHeight="1"/>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>（定義）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>第3条　本規程において「ハラスメント」とは、利用者等の言動により従業員が不快感、屈辱感、恐怖感等を受け、健康や就業環境が害される行為をいう。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>2　ハラスメントには、次の行為を含む。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>（1）身体的暴力</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・殴打、押し倒し、突き飛ばし、掴みかかる行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・物を投げつける、蹴る、刃物等を示すなどの威嚇行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="8" customHeight="1"/>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>（2）精神的暴力</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・大声での罵倒、威嚇、脅迫、恫喝</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・「無能」「役立たず」等の人格を否定する発言</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・差別的言動（国籍、性別、年齢、障害、宗教等に基づくもの）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・過度で不合理な要求、業務妨害となる過剰な干渉</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="8" customHeight="1"/>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>（3）セクシュアル・ハラスメント</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・性的な冗談や発言、卑猥な言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・不必要かつ一方的な身体接触</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・性的関心の示唆、交際の強要</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・性的な言動を拒否したことによる嫌がらせ</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="8" customHeight="1"/>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>（4）ストーカー的言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・訪問や電話、メール等の執拗な繰り返し</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・待ち伏せ、尾行、従業員の私生活への過度な介入</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・個人情報を不当に入手・利用しようとする行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="8" customHeight="1"/>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>（5）業務妨害行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・業務の進行を妨げる過剰な監視、干渉、無理難題の要求</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・正当な理由なく職員の交代を強要すること</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・サービス提供を阻害する虚偽の申し立て</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="8" customHeight="1"/>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>（6）その他社会通念上許容されない行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・常識的に見て従業員の心身に負担を与え、職務遂行を困難にさせる一切の言動</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="8" customHeight="1"/>
+    <row r="66" ht="32" customHeight="1">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>3　「二次被害」とは、被害を申告した従業員に対する詮索、責任転嫁、報復、中傷、孤立化など、被害を拡大・継続させる行為をいう。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="8" customHeight="1"/>
+    <row r="68" ht="48" customHeight="1">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>4　認知症等の病状や障害の特性による言動であっても、従業員の安全確保の対象とする。ただし、その対応にあたっては、利用者の病状等を踏まえ、居宅介護支援事業所（ケアマネジャー）・主治医等と連携してケアの方法を検討する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="10" customHeight="1"/>
+    <row r="70" ht="8" customHeight="1">
+      <c r="A70" s="7" t="inlineStr"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="8" t="n"/>
+      <c r="D70" s="8" t="n"/>
+      <c r="E70" s="8" t="n"/>
+    </row>
+    <row r="71" ht="10" customHeight="1"/>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>第2章　会社の責務</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>（基本方針）</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>第4条　会社は、利用者等からのハラスメントを一切容認しない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>2　会社は、従業員の安全と尊厳を守り、報告を行った者に不利益取扱いをしない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="8" customHeight="1"/>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>（防止責任者および相談窓口）</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>第5条　会社は、ハラスメント防止責任者を設置し、その職務は代表取締役が担う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>2　ハラスメント相談窓口は事業所に設置し、管理者（生田 友哉）が担当する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>3　相談窓口は通報を受けた際、速やかに事実確認・初動対応を行い、防止責任者に報告する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="8" customHeight="1"/>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>（教育・研修）</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>第6条　会社は、従業員に対し、次の措置を講じる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>（1）入社時および年1回のハラスメント防止研修の実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>（2）管理職に対する事案対応力強化研修の実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>（3）利用者・家族に対する契約時の「ハラスメント禁止条項」の説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="8" customHeight="1"/>
+    <row r="88" ht="8" customHeight="1">
+      <c r="A88" s="7" t="inlineStr"/>
+      <c r="B88" s="8" t="n"/>
+      <c r="C88" s="8" t="n"/>
+      <c r="D88" s="8" t="n"/>
+      <c r="E88" s="8" t="n"/>
+    </row>
+    <row r="89" ht="10" customHeight="1"/>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>第3章　従業員の行動指針</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>（発生時の対応）</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="32" customHeight="1">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>第7条　従業員は、利用者等からのハラスメントを受けた場合には、自身の安全を最優先とし、速やかに退避または制止の意思表示を行う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>2　緊急の危険がある場合は、直ちに110番通報等を行うことができる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>3　従業員は、発生から15分以内にサービス提供責任者または管理者へ連絡するものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="8" customHeight="1"/>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>（報告義務）</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>第8条　従業員は、当日中に必ず口頭で報告しなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>2　管理者は、当日中に職員の安全確認と精神的ケアを実施し、サービス継続可否を即断する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="32" customHeight="1">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>3　被害を受けた従業員は、24時間以内に「ハラスメント報告書」を提出する。ただし、心身の状況により困難な場合は、管理者が聞き取りにより作成する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="8" customHeight="1"/>
+    <row r="101" ht="8" customHeight="1">
+      <c r="A101" s="7" t="inlineStr"/>
+      <c r="B101" s="8" t="n"/>
+      <c r="C101" s="8" t="n"/>
+      <c r="D101" s="8" t="n"/>
+      <c r="E101" s="8" t="n"/>
+    </row>
+    <row r="102" ht="10" customHeight="1"/>
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>第4章　会社の対応</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>（調査）</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="20" customHeight="1">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>第9条　防止責任者（代表取締役）は、報告を受けた場合、3日以内に事実確認を行う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="32" customHeight="1">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>2　調査は、被害職員のヒアリング、同席者・目撃者の聴取、ケアマネジャーへの報告、利用者・家族への確認（安全な場合に限る）等を含む。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>3　利用者側には必要に応じて弁明機会を与える。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="8" customHeight="1"/>
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>（レベル判定と対応）</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>第10条　防止責任者は調査後、直ちに以下の区分に基づき対応を決定する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>1　レベル1（軽度）：注意指導で改善可能な場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・利用者・家族へ書面での注意・改善要請</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・ケアマネジャーへの情報提供</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・1か月後の状況確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="20" customHeight="1">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>2　レベル2（中度）：条件付きでサービス継続可能な場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="20" customHeight="1">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・複数職員での訪問を義務化（必要に応じて2人訪問の算定について利用者の同意を得る）</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="20" customHeight="1">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・サービス時間短縮等の条件変更</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="20" customHeight="1">
+      <c r="A118" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・月1回の状況確認とケアマネ連携強化</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="20" customHeight="1">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>3　レベル3（重度）：サービス継続不能と判断される場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="20" customHeight="1">
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・契約解除通知（契約書の定めによる予告期間と引継ぎ期間を考慮）</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="20" customHeight="1">
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・警察への被害相談・通報</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="32" customHeight="1">
+      <c r="A122" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・ケアマネジャー・地域包括支援センター・大阪市と連携した他事業所紹介等、利用者への配慮措置</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="20" customHeight="1">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・代表取締役への緊急報告</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="8" customHeight="1"/>
+    <row r="125" ht="8" customHeight="1">
+      <c r="A125" s="7" t="inlineStr"/>
+      <c r="B125" s="8" t="n"/>
+      <c r="C125" s="8" t="n"/>
+      <c r="D125" s="8" t="n"/>
+      <c r="E125" s="8" t="n"/>
+    </row>
+    <row r="126" ht="10" customHeight="1"/>
+    <row r="127" ht="30" customHeight="1">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>第5章　被害職員の保護・支援</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="20" customHeight="1">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>（医療・精神的支援）</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="32" customHeight="1">
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>第11条　会社は、被害職員に対し、医療機関・カウンセリングの利用を支援し、費用について必要な配慮を行う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="20" customHeight="1">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>2　会社は、被害職員の心身の健康状態を継続的に確認する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="20" customHeight="1">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>3　会社は、労災申請を含む必要な法的手続を支援する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="8" customHeight="1"/>
+    <row r="133" ht="20" customHeight="1">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>（職場環境の配慮）</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="20" customHeight="1">
+      <c r="A134" s="6" t="inlineStr">
+        <is>
+          <t>第12条　会社は、被害職員の希望を尊重し、担当変更や休養措置を講じることができる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="20" customHeight="1">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>2　会社は、不利益取扱いの禁止を明確にし、必要に応じて文書で確約する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="20" customHeight="1">
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>3　会社は、職場復帰に際し、フォロー体制を整備する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="8" customHeight="1"/>
+    <row r="138" ht="8" customHeight="1">
+      <c r="A138" s="7" t="inlineStr"/>
+      <c r="B138" s="8" t="n"/>
+      <c r="C138" s="8" t="n"/>
+      <c r="D138" s="8" t="n"/>
+      <c r="E138" s="8" t="n"/>
+    </row>
+    <row r="139" ht="10" customHeight="1"/>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>第6章　再発防止・改善</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="20" customHeight="1">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>（社内対応）</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="20" customHeight="1">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>第13条　会社は、匿名化した事例を四半期ごとの社内研修で共有し、再発防止を図る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="8" customHeight="1"/>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>（利用者・家族への対応）</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="20" customHeight="1">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>第14条　会社は、利用者・家族に対し、定期的にハラスメント防止の啓発文書を配布する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="8" customHeight="1"/>
+    <row r="147" ht="20" customHeight="1">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>（代表取締役への報告）</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="20" customHeight="1">
+      <c r="A148" s="6" t="inlineStr">
+        <is>
+          <t>第15条　レベル3に該当する案件については、代表取締役が再発防止策を決定する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="8" customHeight="1"/>
+    <row r="150" ht="8" customHeight="1">
+      <c r="A150" s="7" t="inlineStr"/>
+      <c r="B150" s="8" t="n"/>
+      <c r="C150" s="8" t="n"/>
+      <c r="D150" s="8" t="n"/>
+      <c r="E150" s="8" t="n"/>
+    </row>
+    <row r="151" ht="10" customHeight="1"/>
+    <row r="152" ht="30" customHeight="1">
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>第7章　外部対応</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="20" customHeight="1">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>（行政への報告・相談）</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="20" customHeight="1">
+      <c r="A154" s="6" t="inlineStr">
+        <is>
+          <t>第16条　会社は、重大事案について大阪市（保険者）に速やかに報告・相談する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="8" customHeight="1"/>
+    <row r="156" ht="20" customHeight="1">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>（外部への説明）</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="20" customHeight="1">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>第17条　会社は、社会的影響が大きい場合は、代表取締役が適切な外部説明を行う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="8" customHeight="1"/>
+    <row r="159" ht="8" customHeight="1">
+      <c r="A159" s="7" t="inlineStr"/>
+      <c r="B159" s="8" t="n"/>
+      <c r="C159" s="8" t="n"/>
+      <c r="D159" s="8" t="n"/>
+      <c r="E159" s="8" t="n"/>
+    </row>
+    <row r="160" ht="10" customHeight="1"/>
+    <row r="161" ht="30" customHeight="1">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>第8章　雑則</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="20" customHeight="1">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>（マニュアルとの関係）</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="32" customHeight="1">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
+          <t>第18条　本規程に基づく具体的な対応手順は、別途定める「利用者等からのハラスメント防止・対応マニュアル」に従う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="8" customHeight="1"/>
+    <row r="165" ht="8" customHeight="1">
+      <c r="A165" s="7" t="inlineStr"/>
+      <c r="B165" s="8" t="n"/>
+      <c r="C165" s="8" t="n"/>
+      <c r="D165" s="8" t="n"/>
+      <c r="E165" s="8" t="n"/>
+    </row>
+    <row r="166" ht="10" customHeight="1"/>
+    <row r="167" ht="30" customHeight="1">
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>附則</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="20" customHeight="1">
+      <c r="A168" s="6" t="inlineStr">
+        <is>
+          <t>1　本規程の改廃その他定めのない事項は、代表取締役の決定その他関係規程による。</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="20" customHeight="1">
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>2　本規程は令和8年2月1日から施行する。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="114">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A142:E142"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A94:E94"/>
+    <mergeCell ref="A103:E103"/>
+    <mergeCell ref="A168:E168"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A128:E128"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A136:E136"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A113:E113"/>
+    <mergeCell ref="A129:E129"/>
+    <mergeCell ref="A91:E91"/>
+    <mergeCell ref="A131:E131"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A156:E156"/>
+    <mergeCell ref="A165:E165"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A115:E115"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A130:E130"/>
+    <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A83:E83"/>
+    <mergeCell ref="A148:E148"/>
+    <mergeCell ref="A157:E157"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A138:E138"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A119:E119"/>
+    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A118:E118"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A133:E133"/>
+    <mergeCell ref="A80:E80"/>
+    <mergeCell ref="A120:E120"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A104:E104"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A159:E159"/>
+    <mergeCell ref="A97:E97"/>
+    <mergeCell ref="A106:E106"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A147:E147"/>
+    <mergeCell ref="A161:E161"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A123:E123"/>
+    <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A86:E86"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A141:E141"/>
+    <mergeCell ref="A135:E135"/>
+    <mergeCell ref="A150:E150"/>
+    <mergeCell ref="A144:E144"/>
+    <mergeCell ref="A122:E122"/>
+    <mergeCell ref="A125:E125"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A134:E134"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A152:E152"/>
+    <mergeCell ref="A121:E121"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A127:E127"/>
+    <mergeCell ref="A167:E167"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A114:E114"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A98:E98"/>
+    <mergeCell ref="A169:E169"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A107:E107"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A88:E88"/>
+    <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A153:E153"/>
+    <mergeCell ref="A162:E162"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="A99:E99"/>
+    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A145:E145"/>
+    <mergeCell ref="A154:E154"/>
+    <mergeCell ref="A163:E163"/>
+    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A116:E116"/>
+    <mergeCell ref="A140:E140"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A109:E109"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A117:E117"/>
+    <mergeCell ref="A111:E111"/>
+    <mergeCell ref="A92:E92"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;9 株式会社dhpケアマネジメント　いいかいご　利用者等からのハラスメント防止・対応規程</oddHeader>
+    <oddFooter>&amp;C&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="25" min="0" max="16383" man="1"/>
+  </rowBreaks>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E138"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>株式会社dhpケアマネジメント　いいかいご</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1"/>
+    <row r="3" ht="24" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1"/>
+    <row r="5" ht="24" customHeight="1"/>
+    <row r="6" ht="24" customHeight="1"/>
+    <row r="7" ht="24" customHeight="1"/>
+    <row r="8" ht="24" customHeight="1"/>
+    <row r="9" ht="24" customHeight="1"/>
+    <row r="10" ht="24" customHeight="1"/>
+    <row r="11" ht="24" customHeight="1"/>
+    <row r="12" ht="24" customHeight="1"/>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>利用者等からのハラスメント
+防止・対応マニュアル</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1"/>
+    <row r="15" ht="24" customHeight="1"/>
+    <row r="16" ht="24" customHeight="1"/>
+    <row r="17" ht="24" customHeight="1"/>
+    <row r="18" ht="24" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1"/>
+    <row r="21" ht="24" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1"/>
+    <row r="23" ht="24" customHeight="1"/>
+    <row r="24" ht="24" customHeight="1"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>施行　令和8年2月1日</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>1．本マニュアルの位置づけ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　1．本マニュアルは「利用者等からのハラスメント防止・対応規程」に基づき、従業員が現場で直面した際に適切かつ迅速に対応するための具体的手順を示す。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　2．規程が「会社としての方針・責任体制」を定めるのに対し、本マニュアルは「現場職員の実務行動指針」として機能する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3．本マニュアルは全従業員（登録ヘルパーを含む）に周知し、常に最新の知見・事例に基づき改訂される。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="8" customHeight="1"/>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>2．発生時の現場対応</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>2-1．即時退避判断基準</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>以下に該当する場合は、原則として即座に退避する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・身体への接触や暴力の兆候</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・性的発言・行為・身体接触</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・大声での威嚇・恫喝・暴言</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・物を投げる等の威嚇行為</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・継続的な人格否定発言</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="8" customHeight="1"/>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>2-2．現場での行動手順</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・「困ります、やめてください」と明確に制止。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・継続する場合は即座に退避、安全な場所へ移動。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・利用者に急変等の危険がある場合は、退避後に管理者・家族・ケアマネジャーへ連絡し、安全確認の方法を相談する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・生命の危険を感じた場合は110番通報、負傷時は119番通報。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・15分以内にサービス提供責任者→管理者へ電話連絡。</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・可能であれば音声録音・写真撮影等で証拠を保全（安全確保優先）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="8" customHeight="1"/>
+    <row r="48" ht="26" customHeight="1">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>3．第一報・初期対応（当日中）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>3-1．職員の第一報</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・発生直後にサービス提供責任者へ報告。</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・その後、管理者へ報告。</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="8" customHeight="1"/>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>3-2．管理者の初期対応</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・職員の安全確認と精神的ケア。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・当日のサービス継続可否を即断（安全第一原則）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・代替職員手配またはサービス停止の判断（停止する場合はケアマネジャーへ連絡）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・24時間以内に「ハラスメント報告書」作成を依頼。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・証拠（音声・写真・目撃証言・診断書等）の有無を確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・報告内容を代表取締役へ送付。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="8" customHeight="1"/>
+    <row r="61" ht="26" customHeight="1">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>4．事実確認・調査（3日以内）</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・調査主体：代表取締役（防止責任者）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・被害職員への詳細ヒアリング（録音・記録）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・同席者・目撃者の事情聴取。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・ケアマネジャーへの状況報告・情報収集。</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・利用者・家族への事実確認（安全な場合に限る）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・利用者側への弁明機会の提供。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・結果は「調査報告書」にまとめ、防止責任者が対応レベルを判定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="8" customHeight="1"/>
+    <row r="70" ht="26" customHeight="1">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>5．レベル判定と対応決定（調査完了後即時）</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>レベル1（軽度）：注意指導で改善可能</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・利用者・家族へ書面での注意・改善要請。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・ケアマネジャーへの情報提供。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・1か月後の状況確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="8" customHeight="1"/>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>レベル2（中度）：条件付きサービス継続</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・複数職員での訪問を義務化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・サービス時間短縮等の条件変更。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・月1回の状況確認とケアマネジャー連携。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="8" customHeight="1"/>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>レベル3（重度）：契約解除・警察対応</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・契約解除通知（契約書の予告期間と引継ぎ期間を確保）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・警察への相談・通報。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・ケアマネジャー・地域包括支援センターと連携した他事業所紹介等、利用者への配慮措置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・代表取締役への緊急報告。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="8" customHeight="1"/>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="15" t="inlineStr">
+        <is>
+          <t>6．被害職員の保護・支援（全レベル共通）</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="16" t="inlineStr">
+        <is>
+          <t>医療・精神的支援</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・医療機関・カウンセリングの案内と費用支援。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・定期的な心身健康確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・労災申請支援と必要書類作成協力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="8" customHeight="1"/>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="16" t="inlineStr">
+        <is>
+          <t>職場環境の配慮</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・担当変更・休養措置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・不利益取扱い禁止を文書で確約。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・職場復帰時のフォロー体制を整備。</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="8" customHeight="1"/>
+    <row r="98" ht="26" customHeight="1">
+      <c r="A98" s="15" t="inlineStr">
+        <is>
+          <t>7．再発防止・継続改善</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・匿名化事例の社内研修での共有。</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・四半期ごとの「ハラスメント事例検討会」を開催。</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・利用者・家族への啓発文書を定期配布。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・レベル3案件は代表取締役が再発防止策を決定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・年度末に「ハラスメント対応年次報告書」を作成し、代表取締役に提出。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="8" customHeight="1"/>
+    <row r="105" ht="26" customHeight="1">
+      <c r="A105" s="15" t="inlineStr">
+        <is>
+          <t>8．記録・報告・保管</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="20" customHeight="1">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・報告書、調査報告書、証拠資料は管理者が一元管理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・保存期間は原則5年間とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・個人情報は個人情報保護法および「情報管理規程」に基づき厳格に管理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="8" customHeight="1"/>
+    <row r="110" ht="26" customHeight="1">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>9．改訂・見直し</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="32" customHeight="1">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・本マニュアルは、法令改正、行政指導、判例、社会情勢、実際の事案発生状況等を踏まえ、適宜改訂する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・改訂は管理者が案を作成し、防止責任者（代表取締役）が承認する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・改訂版は全従業員に速やかに周知する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="8" customHeight="1"/>
+    <row r="115" ht="26" customHeight="1">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>10．参考：対応フロー（図解）</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="10" customHeight="1"/>
+    <row r="117" ht="26" customHeight="1">
+      <c r="B117" s="17" t="inlineStr">
+        <is>
+          <t>発生</t>
+        </is>
+      </c>
+      <c r="C117" s="22" t="n"/>
+      <c r="D117" s="22" t="n"/>
+    </row>
+    <row r="118" ht="16" customHeight="1">
+      <c r="C118" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="26" customHeight="1">
+      <c r="B119" s="17" t="inlineStr">
+        <is>
+          <t>退避・制止（困ります、やめてください）</t>
+        </is>
+      </c>
+      <c r="C119" s="22" t="n"/>
+      <c r="D119" s="22" t="n"/>
+    </row>
+    <row r="120" ht="16" customHeight="1">
+      <c r="C120" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="26" customHeight="1">
+      <c r="B121" s="17" t="inlineStr">
+        <is>
+          <t>110番／119番（必要時）</t>
+        </is>
+      </c>
+      <c r="C121" s="22" t="n"/>
+      <c r="D121" s="22" t="n"/>
+    </row>
+    <row r="122" ht="16" customHeight="1">
+      <c r="C122" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="26" customHeight="1">
+      <c r="B123" s="17" t="inlineStr">
+        <is>
+          <t>15分以内にサービス提供責任者・管理者へ報告</t>
+        </is>
+      </c>
+      <c r="C123" s="22" t="n"/>
+      <c r="D123" s="22" t="n"/>
+    </row>
+    <row r="124" ht="16" customHeight="1">
+      <c r="C124" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="26" customHeight="1">
+      <c r="B125" s="17" t="inlineStr">
+        <is>
+          <t>当日中：管理者が安全確認・サービス可否判断</t>
+        </is>
+      </c>
+      <c r="C125" s="22" t="n"/>
+      <c r="D125" s="22" t="n"/>
+    </row>
+    <row r="126" ht="16" customHeight="1">
+      <c r="C126" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="26" customHeight="1">
+      <c r="B127" s="17" t="inlineStr">
+        <is>
+          <t>24時間以内：報告書作成・証拠確認</t>
+        </is>
+      </c>
+      <c r="C127" s="22" t="n"/>
+      <c r="D127" s="22" t="n"/>
+    </row>
+    <row r="128" ht="16" customHeight="1">
+      <c r="C128" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="26" customHeight="1">
+      <c r="B129" s="17" t="inlineStr">
+        <is>
+          <t>3日以内：代表取締役が調査・弁明機会付与</t>
+        </is>
+      </c>
+      <c r="C129" s="22" t="n"/>
+      <c r="D129" s="22" t="n"/>
+    </row>
+    <row r="130" ht="16" customHeight="1">
+      <c r="C130" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="26" customHeight="1">
+      <c r="B131" s="17" t="inlineStr">
+        <is>
+          <t>レベル判定（1：注意／2：条件付継続／3：契約解除・警察）</t>
+        </is>
+      </c>
+      <c r="C131" s="22" t="n"/>
+      <c r="D131" s="22" t="n"/>
+    </row>
+    <row r="132" ht="16" customHeight="1">
+      <c r="C132" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="26" customHeight="1">
+      <c r="B133" s="17" t="inlineStr">
+        <is>
+          <t>被害職員支援（医療・休養・労災・不利益禁止）</t>
+        </is>
+      </c>
+      <c r="C133" s="22" t="n"/>
+      <c r="D133" s="22" t="n"/>
+    </row>
+    <row r="134" ht="16" customHeight="1">
+      <c r="C134" s="18" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="26" customHeight="1">
+      <c r="B135" s="17" t="inlineStr">
+        <is>
+          <t>再発防止（研修・事例検討会・代表取締役への報告）</t>
+        </is>
+      </c>
+      <c r="C135" s="22" t="n"/>
+      <c r="D135" s="22" t="n"/>
+    </row>
+    <row r="136" ht="10" customHeight="1"/>
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>＜附則＞</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="20" customHeight="1">
+      <c r="A138" s="6" t="inlineStr">
+        <is>
+          <t>本マニュアルは、令和8年2月1日から施行する。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="91">
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A94:E94"/>
+    <mergeCell ref="A103:E103"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A87:E87"/>
+    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A137:E137"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A89:E89"/>
+    <mergeCell ref="B133:D133"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A113:E113"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="B135:D135"/>
+    <mergeCell ref="B125:D125"/>
+    <mergeCell ref="A91:E91"/>
+    <mergeCell ref="A100:E100"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A115:E115"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A83:E83"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A138:E138"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A95:E95"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A106:E106"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A108:E108"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="B123:D123"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="B117:D117"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A98:E98"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A107:E107"/>
+    <mergeCell ref="B119:D119"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A88:E88"/>
+    <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="B127:D127"/>
+    <mergeCell ref="A99:E99"/>
+    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A76:E76"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="B129:D129"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="B121:D121"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A62:E62"/>
+    <mergeCell ref="B131:D131"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A102:E102"/>
+    <mergeCell ref="A111:E111"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;9 株式会社dhpケアマネジメント　いいかいご　利用者等からのハラスメント防止・対応マニュアル</oddHeader>
+    <oddFooter>&amp;C&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="25" min="0" max="16383" man="1"/>
+    <brk id="114" min="0" max="16383" man="1"/>
+  </rowBreaks>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
運営規程: align hours, area, fees and staffing with 重要事項説明書
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_社内規程一式.xlsx
+++ b/output/いいかいご_社内規程一式.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -816,7 +816,7 @@
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>（3）訪問介護員　3名以上（常勤換算2.5名以上）</t>
+          <t>（3）訪問介護員　10名（常勤7名、非常勤3名）（常勤換算2.5名以上を確保する）</t>
         </is>
       </c>
     </row>
@@ -830,14 +830,14 @@
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>（4）事務職員　0名（常勤又は非常勤 0名）</t>
+          <t>（4）事務職員　1名（常勤1名）</t>
         </is>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　　必要な事務を行う。</t>
+          <t xml:space="preserve">　　介護給付費等の請求事務及び通信連絡事務等を行う。</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>（1）営業日　月曜日から日曜日までとする。ただし、祝日、12月30日から1月3日までを除く。</t>
+          <t>（1）営業日　月曜日から金曜日までとする。ただし、祝日、8月13日から8月15日まで、12月30日から1月3日までを除く。</t>
         </is>
       </c>
     </row>
@@ -873,416 +873,423 @@
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>（3）サービス提供時間　24時間（午前0時から午後12時まで）とする。</t>
+          <t>（3）サービス提供日　1月1日から1月3日までを除く毎日とする。</t>
         </is>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>（4）営業時間外は電話等により常時連絡が可能な体制とする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="8" customHeight="1"/>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="4" t="inlineStr">
+          <t>（4）サービス提供時間　午前7時から午後11時までとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>（5）営業時間外のサービス提供時間帯は、電話等により連絡が可能な体制とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="8" customHeight="1"/>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>（指定訪問介護の内容）</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>第7条　事業所で行う指定訪問介護の内容は次のとおりとする。</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
+          <t>第7条　事業所で行う指定訪問介護の内容は次のとおりとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
           <t>（1）訪問介護計画の作成</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="32" customHeight="1">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>（2）身体介護に関する内容　①排泄・食事介助 ②清拭・入浴・身体整容 ③体位変換 ④移動・移乗介助、外出介助 ⑤その他の必要な身体の介護</t>
         </is>
       </c>
     </row>
     <row r="70" ht="32" customHeight="1">
       <c r="A70" s="5" t="inlineStr">
         <is>
+          <t>（2）身体介護に関する内容　①排泄・食事介助 ②清拭・入浴・身体整容 ③体位変換 ④移動・移乗介助、外出介助 ⑤その他の必要な身体の介護</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="32" customHeight="1">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
           <t>（3）生活援助に関する内容　①調理 ②衣類の洗濯、補修 ③住居の掃除、整理整頓 ④生活必需品の買い物 ⑤その他必要な家事</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="8" customHeight="1"/>
-    <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="4" t="inlineStr">
+    <row r="72" ht="8" customHeight="1"/>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>（指定訪問介護の利用料等）</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="64" customHeight="1">
-      <c r="A73" s="5" t="inlineStr">
+    <row r="74" ht="64" customHeight="1">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>第8条　指定訪問介護を提供した場合の利用料の額は、介護報酬告示上の額とし、そのサービスが法定代理受領サービスであるときは、利用料のうち各利用者の負担割合に応じた額の支払いを受けるものとする。なお、法定代理受領以外の利用料については、「指定居宅サービスに要する費用の額の算定に関する基準」（平成12年2月10日厚生省告示第19号）によるものとする。</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="32" customHeight="1">
-      <c r="A74" s="5" t="inlineStr">
+    <row r="75" ht="32" customHeight="1">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>2　次条に定める通常の事業の実施地域を越えて行う事業に要する交通費は、その実費を徴収する。なお、自動車を使用した場合の交通費は、次の額とする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="5" t="inlineStr">
-        <is>
-          <t>（1）事業所から片道5キロメートル未満　100円（税別）</t>
         </is>
       </c>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>（2）事業所から片道5キロメートル以上　1kmを増すごとに20円ずつ加算（税別）</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="32" customHeight="1">
+          <t>（1）事業所から片道5キロメートル未満　200円</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1">
       <c r="A77" s="5" t="inlineStr">
         <is>
+          <t>（2）事業所から片道5キロメートル以上　500円</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="32" customHeight="1">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
           <t>3　前2項の利用料等の支払を受けたときは、利用者又はその家族に対し、利用料とその他の利用料（個別の費用ごとに区分したもの）について記載した領収書を交付する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="48" customHeight="1">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>4　指定訪問介護の提供の開始に際しては、あらかじめ、利用者又はその家族に対し、当該サービスの内容及び費用に関し事前に文書で説明した上で、その内容及び支払いに同意する旨の文書に署名（記名押印）を受けるものとする。</t>
         </is>
       </c>
     </row>
     <row r="79" ht="48" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
         <is>
+          <t>4　指定訪問介護の提供の開始に際しては、あらかじめ、利用者又はその家族に対し、当該サービスの内容及び費用に関し事前に文書で説明した上で、その内容及び支払いに同意する旨の文書に署名（記名押印）を受けるものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="48" customHeight="1">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
           <t>5　法定代理受領サービスに該当しない指定訪問介護に係る利用料の支払いを受けたときは、提供した指定訪問介護の内容、費用の額その他必要と認められる事項を記載したサービス提供証明書を利用者に対して交付するものとする。</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="8" customHeight="1"/>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="4" t="inlineStr">
+    <row r="81" ht="8" customHeight="1"/>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>（通常の事業の実施地域）</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="5" t="inlineStr">
-        <is>
-          <t>第9条　通常の事業の実施地域は、大阪市とする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="8" customHeight="1"/>
-    <row r="84" ht="20" customHeight="1">
-      <c r="A84" s="4" t="inlineStr">
+    <row r="83" ht="32" customHeight="1">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>第9条　通常の事業の実施地域は、大阪市西淀川区、淀川区、東淀川区、天王寺区、中央区、北区とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="8" customHeight="1"/>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>（衛生管理等）</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="32" customHeight="1">
-      <c r="A85" s="5" t="inlineStr">
-        <is>
-          <t>第10条　訪問介護員等の清潔の保持及び健康状態の管理を行うとともに、事業所の設備及び備品等の衛生的な管理に努めるものとする。</t>
         </is>
       </c>
     </row>
     <row r="86" ht="32" customHeight="1">
       <c r="A86" s="5" t="inlineStr">
         <is>
+          <t>第10条　訪問介護員等の清潔の保持及び健康状態の管理を行うとともに、事業所の設備及び備品等の衛生的な管理に努めるものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="32" customHeight="1">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
           <t>2　事業所は、感染症の予防及びまん延の防止のため、感染対策委員会の開催（おおむね6か月に1回以上）、指針の整備、研修及び訓練の実施を行う。</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="8" customHeight="1"/>
-    <row r="88" ht="20" customHeight="1">
-      <c r="A88" s="4" t="inlineStr">
+    <row r="88" ht="8" customHeight="1"/>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
         <is>
           <t>（緊急時等における対応方法）</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="48" customHeight="1">
-      <c r="A89" s="5" t="inlineStr">
+    <row r="90" ht="48" customHeight="1">
+      <c r="A90" s="5" t="inlineStr">
         <is>
           <t>第11条　訪問介護員等は、指定訪問介護の提供を行っているときに利用者に病状の急変、その他緊急事態が生じたときは、速やかに主治医に連絡する等の措置を講じるとともに、管理者に報告する。また、主治医への連絡が困難な場合は、緊急搬送等の必要な措置を講じるものとする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="32" customHeight="1">
-      <c r="A90" s="5" t="inlineStr">
-        <is>
-          <t>2　指定訪問介護の提供により事故が発生した場合は、利用者の所在する市町村、利用者の家族、利用者に係る居宅介護支援事業者等に連絡するとともに、必要な措置を講じるものとする。</t>
         </is>
       </c>
     </row>
     <row r="91" ht="32" customHeight="1">
       <c r="A91" s="5" t="inlineStr">
         <is>
+          <t>2　指定訪問介護の提供により事故が発生した場合は、利用者の所在する市町村、利用者の家族、利用者に係る居宅介護支援事業者等に連絡するとともに、必要な措置を講じるものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="32" customHeight="1">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
           <t>3　利用者に対する指定訪問介護の提供により賠償すべき事故が発生した場合には、損害賠償を速やかに行うものとする。</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="8" customHeight="1"/>
-    <row r="93" ht="20" customHeight="1">
-      <c r="A93" s="4" t="inlineStr">
+    <row r="93" ht="8" customHeight="1"/>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>（苦情処理）</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="32" customHeight="1">
-      <c r="A94" s="5" t="inlineStr">
+    <row r="95" ht="32" customHeight="1">
+      <c r="A95" s="5" t="inlineStr">
         <is>
           <t>第12条　指定訪問介護の提供に係る利用者及びその家族からの苦情に迅速かつ適切に対応するために必要な措置を講じるものとする。</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="64" customHeight="1">
-      <c r="A95" s="5" t="inlineStr">
+    <row r="96" ht="64" customHeight="1">
+      <c r="A96" s="5" t="inlineStr">
         <is>
           <t>2　事業所は、提供した指定訪問介護に関し、介護保険法第23条の規定により市町村が行う文書その他の物件の提出若しくは提示の求め又は当該市町村の職員からの質問若しくは照会に応じ、及び市町村が行う調査に協力するとともに、市町村から指導又は助言を受けた場合は、当該指導又は助言に従って必要な改善を行うものとする。</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="48" customHeight="1">
-      <c r="A96" s="5" t="inlineStr">
+    <row r="97" ht="48" customHeight="1">
+      <c r="A97" s="5" t="inlineStr">
         <is>
           <t>3　事業所は、提供した指定訪問介護に係る利用者からの苦情に関して国民健康保険団体連合会が行う調査に協力するとともに、国民健康保険団体連合会から指導又は助言を受けた場合は、当該指導又は助言に従って必要な改善を行うものとする。</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="8" customHeight="1"/>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="4" t="inlineStr">
+    <row r="98" ht="8" customHeight="1"/>
+    <row r="99" ht="20" customHeight="1">
+      <c r="A99" s="4" t="inlineStr">
         <is>
           <t>（個人情報の保護）</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="48" customHeight="1">
-      <c r="A99" s="5" t="inlineStr">
-        <is>
-          <t>第13条　事業所は、利用者の個人情報について「個人情報の保護に関する法律」及び厚生労働省が策定した「医療・介護関係事業者における個人情報の適切な取扱いのためのガイダンス」を遵守し適切な取り扱いに努めるものとする。</t>
         </is>
       </c>
     </row>
     <row r="100" ht="48" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
         <is>
+          <t>第13条　事業所は、利用者の個人情報について「個人情報の保護に関する法律」及び厚生労働省が策定した「医療・介護関係事業者における個人情報の適切な取扱いのためのガイダンス」を遵守し適切な取り扱いに努めるものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="48" customHeight="1">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
           <t>2　事業者が得た利用者又はその家族の個人情報については、事業者での介護サービスの提供以外の目的では原則的に利用しないものとし、外部への情報提供については必要に応じて利用者又はその代理人の了解を得るものとする。</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="8" customHeight="1"/>
-    <row r="102" ht="20" customHeight="1">
-      <c r="A102" s="4" t="inlineStr">
+    <row r="102" ht="8" customHeight="1"/>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="4" t="inlineStr">
         <is>
           <t>（虐待防止に関する事項）</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="20" customHeight="1">
-      <c r="A103" s="5" t="inlineStr">
-        <is>
-          <t>第14条　事業所は、利用者の人権の擁護・虐待等の防止のため次の措置を講ずるものとする。</t>
         </is>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>（1）虐待防止のための対策を検討する委員会の定期的な開催と、その結果の従業者への周知</t>
+          <t>第14条　事業所は、利用者の人権の擁護・虐待等の防止のため次の措置を講ずるものとする。</t>
         </is>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>（2）虐待防止のための指針の整備</t>
+          <t>（1）虐待防止のための対策を検討する委員会の定期的な開催と、その結果の従業者への周知</t>
         </is>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>（3）虐待を防止するための従業者に対する研修の実施（年1回以上及び新規採用時）</t>
+          <t>（2）虐待防止のための指針の整備</t>
         </is>
       </c>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>（4）前3号の措置を適切に実施するための担当者の設置（虐待防止責任者：管理者）</t>
+          <t>（3）虐待を防止するための従業者に対する研修の実施（年1回以上及び新規採用時）</t>
         </is>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>（5）利用者及びその家族からの苦情処理体制の整備</t>
+          <t>（4）前3号の措置を適切に実施するための担当者の設置（虐待防止責任者：管理者）</t>
         </is>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
+          <t>（5）利用者及びその家族からの苦情処理体制の整備</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
           <t>（6）その他虐待防止のために必要な措置</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="48" customHeight="1">
-      <c r="A110" s="5" t="inlineStr">
+    <row r="111" ht="48" customHeight="1">
+      <c r="A111" s="5" t="inlineStr">
         <is>
           <t>2　事業所は、サービス提供中に、当該事業所従業者又は養護者（利用者の家族等高齢者を現に養護する者）による虐待を受けたと思われる利用者を発見した場合は、速やかに、これを市町村に通報するものとする。</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="8" customHeight="1"/>
-    <row r="112" ht="20" customHeight="1">
-      <c r="A112" s="4" t="inlineStr">
+    <row r="112" ht="8" customHeight="1"/>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="4" t="inlineStr">
         <is>
           <t>（身体拘束等の禁止）</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="32" customHeight="1">
-      <c r="A113" s="5" t="inlineStr">
-        <is>
-          <t>第15条　事業所は、利用者又は他の利用者等の生命又は身体を保護するため緊急やむを得ない場合を除き、身体的拘束その他利用者の行動を制限する行為を行わない。</t>
         </is>
       </c>
     </row>
     <row r="114" ht="32" customHeight="1">
       <c r="A114" s="5" t="inlineStr">
         <is>
+          <t>第15条　事業所は、利用者又は他の利用者等の生命又は身体を保護するため緊急やむを得ない場合を除き、身体的拘束その他利用者の行動を制限する行為を行わない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="32" customHeight="1">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
           <t>2　緊急やむを得ず身体的拘束等を行う場合には、その態様及び時間、その際の利用者の心身の状況並びに緊急やむを得ない理由を記録する。</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="8" customHeight="1"/>
-    <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="4" t="inlineStr">
+    <row r="116" ht="8" customHeight="1"/>
+    <row r="117" ht="20" customHeight="1">
+      <c r="A117" s="4" t="inlineStr">
         <is>
           <t>（業務継続計画の策定等）</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="48" customHeight="1">
-      <c r="A117" s="5" t="inlineStr">
+    <row r="118" ht="48" customHeight="1">
+      <c r="A118" s="5" t="inlineStr">
         <is>
           <t>第16条　事業所は、感染症や非常災害の発生時において、利用者に対する指定訪問介護の提供を継続的に実施し、及び非常時の体制で早期の業務再開を図るための業務継続計画を策定し、当該計画に従い必要な措置を講じる。</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="32" customHeight="1">
-      <c r="A118" s="5" t="inlineStr">
+    <row r="119" ht="32" customHeight="1">
+      <c r="A119" s="5" t="inlineStr">
         <is>
           <t>2　事業所は、従業者に対し、業務継続計画について周知するとともに、必要な研修及び訓練を定期的に実施する。</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="8" customHeight="1"/>
-    <row r="120" ht="20" customHeight="1">
-      <c r="A120" s="4" t="inlineStr">
+    <row r="120" ht="8" customHeight="1"/>
+    <row r="121" ht="20" customHeight="1">
+      <c r="A121" s="4" t="inlineStr">
         <is>
           <t>（その他運営に関する重要事項）</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="32" customHeight="1">
-      <c r="A121" s="5" t="inlineStr">
+    <row r="122" ht="32" customHeight="1">
+      <c r="A122" s="5" t="inlineStr">
         <is>
           <t>第17条　事業所は、従業者の資質向上のために次のとおり研修の機会を設けるものとし、また、業務の執行体制についても検証、整備する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="20" customHeight="1">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>（1）採用時研修　採用後1か月以内</t>
         </is>
       </c>
     </row>
     <row r="123" ht="20" customHeight="1">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>（2）継続研修　年2回</t>
+          <t>（1）採用時研修　採用後1か月以内</t>
         </is>
       </c>
     </row>
     <row r="124" ht="20" customHeight="1">
       <c r="A124" s="5" t="inlineStr">
         <is>
+          <t>（2）継続研修　年2回</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
           <t>2　従業者は、業務上知り得た利用者又はその家族の秘密を保持する。</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="48" customHeight="1">
-      <c r="A125" s="5" t="inlineStr">
+    <row r="126" ht="48" customHeight="1">
+      <c r="A126" s="5" t="inlineStr">
         <is>
           <t>3　事業所は、従業者であった者に、業務上知り得た利用者又はその家族の秘密を保持させるため、従業者でなくなった後においてもこれらの秘密を保持するべき旨を、従業者との雇用契約の内容とする。</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="20" customHeight="1">
-      <c r="A126" s="5" t="inlineStr">
+    <row r="127" ht="20" customHeight="1">
+      <c r="A127" s="5" t="inlineStr">
         <is>
           <t>4　事業所は、職場におけるハラスメントの防止のための方針の明確化等の必要な措置を講じる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="32" customHeight="1">
-      <c r="A127" s="5" t="inlineStr">
-        <is>
-          <t>5　事業所は、指定訪問介護に関する諸記録を整備し、そのサービス提供をした日から最低5年間は保存するものとする。</t>
         </is>
       </c>
     </row>
     <row r="128" ht="32" customHeight="1">
       <c r="A128" s="5" t="inlineStr">
         <is>
+          <t>5　事業所は、指定訪問介護に関する諸記録を整備し、そのサービス提供をした日から最低5年間は保存するものとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="32" customHeight="1">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
           <t>6　この規程に定める事項の外、運営に関する重要事項は株式会社dhpケアマネジメントと事業所の管理者との協議に基づいて定めるものとする。</t>
         </is>
       </c>
     </row>
-    <row r="129" ht="8" customHeight="1"/>
-    <row r="130" ht="20" customHeight="1">
-      <c r="A130" s="4" t="inlineStr">
+    <row r="130" ht="8" customHeight="1"/>
+    <row r="131" ht="20" customHeight="1">
+      <c r="A131" s="4" t="inlineStr">
         <is>
           <t>附則</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="20" customHeight="1">
-      <c r="A131" s="5" t="inlineStr">
+    <row r="132" ht="20" customHeight="1">
+      <c r="A132" s="5" t="inlineStr">
         <is>
           <t>この規程は、令和8年2月1日から施行する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="92">
+  <mergeCells count="93">
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="A1:E1"/>
@@ -1290,6 +1297,8 @@
     <mergeCell ref="A94:E94"/>
     <mergeCell ref="A103:E103"/>
     <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A87:E87"/>
+    <mergeCell ref="A65:E65"/>
     <mergeCell ref="A128:E128"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A46:E46"/>
@@ -1298,29 +1307,33 @@
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A113:E113"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="A129:E129"/>
     <mergeCell ref="A91:E91"/>
     <mergeCell ref="A131:E131"/>
     <mergeCell ref="A100:E100"/>
     <mergeCell ref="A52:E52"/>
     <mergeCell ref="A63:E63"/>
-    <mergeCell ref="A93:E93"/>
-    <mergeCell ref="A130:E130"/>
+    <mergeCell ref="A115:E115"/>
     <mergeCell ref="A77:E77"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A83:E83"/>
     <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A132:E132"/>
     <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A119:E119"/>
     <mergeCell ref="A69:E69"/>
     <mergeCell ref="A78:E78"/>
     <mergeCell ref="A118:E118"/>
     <mergeCell ref="A75:E75"/>
-    <mergeCell ref="A120:E120"/>
+    <mergeCell ref="A80:E80"/>
     <mergeCell ref="A55:E55"/>
     <mergeCell ref="A95:E95"/>
     <mergeCell ref="A104:E104"/>
     <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A97:E97"/>
     <mergeCell ref="A106:E106"/>
     <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A81:E81"/>
     <mergeCell ref="A96:E96"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="A40:E40"/>
@@ -1333,16 +1346,12 @@
     <mergeCell ref="A124:E124"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A108:E108"/>
-    <mergeCell ref="A84:E84"/>
-    <mergeCell ref="A66:E66"/>
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A86:E86"/>
     <mergeCell ref="A42:E42"/>
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="A122:E122"/>
     <mergeCell ref="A125:E125"/>
-    <mergeCell ref="A72:E72"/>
-    <mergeCell ref="A112:E112"/>
     <mergeCell ref="A121:E121"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A44:E44"/>
@@ -1351,11 +1360,9 @@
     <mergeCell ref="A114:E114"/>
     <mergeCell ref="A59:E59"/>
     <mergeCell ref="A64:E64"/>
-    <mergeCell ref="A98:E98"/>
     <mergeCell ref="A51:E51"/>
     <mergeCell ref="A107:E107"/>
     <mergeCell ref="A61:E61"/>
-    <mergeCell ref="A88:E88"/>
     <mergeCell ref="A70:E70"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A41:E41"/>
@@ -1364,17 +1371,18 @@
     <mergeCell ref="A74:E74"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A101:E101"/>
     <mergeCell ref="A76:E76"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A85:E85"/>
-    <mergeCell ref="A116:E116"/>
     <mergeCell ref="A126:E126"/>
     <mergeCell ref="A53:E53"/>
     <mergeCell ref="A109:E109"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A102:E102"/>
     <mergeCell ref="A117:E117"/>
+    <mergeCell ref="A111:E111"/>
+    <mergeCell ref="A92:E92"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update committee member lists (吉田俊輔・吉田麻美・生田友哉・WIN YADANAR AWNG)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_社内規程一式.xlsx
+++ b/output/いいかいご_社内規程一式.xlsx
@@ -139,7 +139,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -156,11 +156,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -244,6 +272,11 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -7292,7 +7325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E142"/>
+  <dimension ref="A1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -8186,124 +8219,104 @@
       </c>
       <c r="D134" s="22" t="inlineStr">
         <is>
-          <t>感染症対策全体の統括・研修・教育担当を兼務</t>
+          <t>感染症対策全体の統括・最終判断・行政報告。研修・教育担当を兼務</t>
         </is>
       </c>
       <c r="E134" s="23" t="n"/>
     </row>
-    <row r="135" ht="20" customHeight="1">
+    <row r="135" ht="32" customHeight="1">
       <c r="A135" s="20" t="inlineStr">
         <is>
-          <t>副委員長（サービス提供責任者）</t>
+          <t>委員（代表取締役）</t>
         </is>
       </c>
       <c r="B135" s="21" t="n"/>
       <c r="C135" s="22" t="inlineStr">
         <is>
-          <t>岩谷</t>
+          <t>吉田 俊輔</t>
         </is>
       </c>
       <c r="D135" s="22" t="inlineStr">
         <is>
-          <t>現場調整・周知・実務統括</t>
+          <t>法人としての方針決定、BCPの承認、重大事案時の対外対応</t>
         </is>
       </c>
       <c r="E135" s="23" t="n"/>
     </row>
-    <row r="136" ht="20" customHeight="1">
+    <row r="136" ht="32" customHeight="1">
       <c r="A136" s="20" t="inlineStr">
         <is>
-          <t>看護職委員</t>
+          <t>委員（事務・総務）</t>
         </is>
       </c>
       <c r="B136" s="21" t="n"/>
       <c r="C136" s="22" t="inlineStr">
         <is>
-          <t>松本</t>
+          <t>吉田 麻美</t>
         </is>
       </c>
       <c r="D136" s="22" t="inlineStr">
         <is>
-          <t>医療的助言・PPE指導</t>
+          <t>議事録作成、記録整備・行政書類確認、衛生用品の在庫管理</t>
         </is>
       </c>
       <c r="E136" s="23" t="n"/>
     </row>
-    <row r="137" ht="20" customHeight="1">
+    <row r="137" ht="32" customHeight="1">
       <c r="A137" s="20" t="inlineStr">
         <is>
-          <t>ヘルパー代表</t>
+          <t>委員（ヘルパー代表）</t>
         </is>
       </c>
       <c r="B137" s="21" t="n"/>
       <c r="C137" s="22" t="inlineStr">
         <is>
-          <t>松川</t>
+          <t>WIN YADANAR AWNG</t>
         </is>
       </c>
       <c r="D137" s="22" t="inlineStr">
         <is>
-          <t>現場情報共有・フィードバック</t>
+          <t>現場情報共有・フィードバック、標準予防策の実施状況の確認</t>
         </is>
       </c>
       <c r="E137" s="23" t="n"/>
     </row>
-    <row r="138" ht="20" customHeight="1">
+    <row r="138" ht="32" customHeight="1">
       <c r="A138" s="20" t="inlineStr">
         <is>
-          <t>事務・総務</t>
+          <t>顧問（任意）</t>
         </is>
       </c>
       <c r="B138" s="21" t="n"/>
       <c r="C138" s="22" t="inlineStr">
         <is>
-          <t>鳥羽</t>
+          <t>主治医・外部専門家・保健所等</t>
         </is>
       </c>
       <c r="D138" s="22" t="inlineStr">
         <is>
-          <t>記録整備・行政書類確認</t>
+          <t>医療的助言・PPE指導（必要に応じて）</t>
         </is>
       </c>
       <c r="E138" s="23" t="n"/>
     </row>
-    <row r="139" ht="20" customHeight="1">
-      <c r="A139" s="20" t="inlineStr">
-        <is>
-          <t>研修・教育担当</t>
-        </is>
-      </c>
-      <c r="B139" s="21" t="n"/>
-      <c r="C139" s="22" t="inlineStr">
-        <is>
-          <t>生田 友哉（兼務）</t>
-        </is>
-      </c>
-      <c r="D139" s="22" t="inlineStr">
-        <is>
-          <t>感染研修の企画・欠席者フォロー</t>
-        </is>
-      </c>
-      <c r="E139" s="23" t="n"/>
-    </row>
-    <row r="140" ht="8" customHeight="1"/>
+    <row r="139" ht="8" customHeight="1"/>
+    <row r="140" ht="20" customHeight="1">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>＜附則＞</t>
+        </is>
+      </c>
+    </row>
     <row r="141" ht="20" customHeight="1">
-      <c r="A141" s="4" t="inlineStr">
-        <is>
-          <t>＜附則＞</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="20" customHeight="1">
-      <c r="A142" s="5" t="inlineStr">
+      <c r="A141" s="5" t="inlineStr">
         <is>
           <t>本資料は、令和8年2月1日から適用する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="107">
-    <mergeCell ref="A142:E142"/>
+  <mergeCells count="105">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A94:E94"/>
     <mergeCell ref="A79:E79"/>
@@ -8342,7 +8355,6 @@
     <mergeCell ref="B53:C53"/>
     <mergeCell ref="A120:E120"/>
     <mergeCell ref="D53:E53"/>
-    <mergeCell ref="A139:B139"/>
     <mergeCell ref="A104:E104"/>
     <mergeCell ref="A32:E32"/>
     <mergeCell ref="A97:E97"/>
@@ -8359,7 +8371,6 @@
     <mergeCell ref="A110:E110"/>
     <mergeCell ref="A124:E124"/>
     <mergeCell ref="B52:C52"/>
-    <mergeCell ref="D139:E139"/>
     <mergeCell ref="D52:E52"/>
     <mergeCell ref="D49:E49"/>
     <mergeCell ref="A25:E25"/>
@@ -8400,6 +8411,7 @@
     <mergeCell ref="D137:E137"/>
     <mergeCell ref="A135:B135"/>
     <mergeCell ref="A126:E126"/>
+    <mergeCell ref="A140:E140"/>
     <mergeCell ref="A109:E109"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A134:B134"/>
@@ -10782,7 +10794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E148"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -11071,489 +11083,503 @@
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　・代表取締役（法人代表者）　吉田 駿成</t>
+          <t xml:space="preserve">　・管理者（委員長）　生田 友哉</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　・管理者（委員長）　生田 友哉</t>
+          <t xml:space="preserve">　・代表取締役（法人代表者）　吉田 俊輔</t>
         </is>
       </c>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　・必要に応じて、サービス提供責任者・担当訪問介護員等の参加を求める</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="8" customHeight="1"/>
+          <t xml:space="preserve">　・事務・総務　吉田 麻美</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・訪問介護員（ヘルパー代表）　WIN YADANAR AWNG</t>
+        </is>
+      </c>
+    </row>
     <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="4" t="inlineStr">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　・必要に応じて、担当訪問介護員・ケアマネジャー・主治医等の参加を求める</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="8" customHeight="1"/>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>③ 委員会の開催</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="48" customHeight="1">
-      <c r="A72" s="5" t="inlineStr">
+    <row r="74" ht="48" customHeight="1">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>年1回以上定期的に開催するほか、必要時に随時開催します。開催はテレビ電話装置等を活用して行うことができ、虐待防止委員会等と一体的に開催することを妨げません。結果は記録し、全職員に周知します。</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="10" customHeight="1"/>
-    <row r="74" ht="26" customHeight="1">
-      <c r="A74" s="16" t="inlineStr">
+    <row r="75" ht="10" customHeight="1"/>
+    <row r="76" ht="26" customHeight="1">
+      <c r="A76" s="16" t="inlineStr">
         <is>
           <t>4．やむを得ず身体拘束を行う場合の対応</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="32" customHeight="1">
-      <c r="A75" s="5" t="inlineStr">
+    <row r="77" ht="32" customHeight="1">
+      <c r="A77" s="5" t="inlineStr">
         <is>
           <t>本人又は他の利用者等の生命又は身体を保護するための措置として、緊急やむを得ず身体拘束を行わなければならない場合は、以下の手順に従って実施します。</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="6" customHeight="1"/>
-    <row r="77" ht="20" customHeight="1">
-      <c r="A77" s="4" t="inlineStr">
+    <row r="78" ht="6" customHeight="1"/>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>1）カンファレンスの実施</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="48" customHeight="1">
-      <c r="A78" s="5" t="inlineStr">
+    <row r="80" ht="48" customHeight="1">
+      <c r="A80" s="5" t="inlineStr">
         <is>
           <t>緊急やむを得ない状況になった場合、委員会の構成員が集まり、拘束による利用者の心身の損害や拘束をしない場合のリスクについて検討し、身体拘束を行う事を選択する前に①切迫性②非代替性③一時性の3要件全てを満たしているかどうかについて検討、確認します。</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="64" customHeight="1">
-      <c r="A79" s="5" t="inlineStr">
+    <row r="81" ht="64" customHeight="1">
+      <c r="A81" s="5" t="inlineStr">
         <is>
           <t>要件を検討・確認した上で、身体拘束を行うことを選択した場合は、拘束の方法、場所、時間帯、期間等について検討し、本人・家族に対する説明書を作成します。また、廃止に向けた取り組み改善の検討会を早急に行い実施に努めます。居宅介護支援事業所（ケアマネジャー）にも報告し、ケアプランへの位置づけについて協議します。</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="6" customHeight="1"/>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="4" t="inlineStr">
+    <row r="82" ht="6" customHeight="1"/>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>2）利用者本人や家族に対しての説明</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="32" customHeight="1">
-      <c r="A82" s="5" t="inlineStr">
+    <row r="84" ht="32" customHeight="1">
+      <c r="A84" s="5" t="inlineStr">
         <is>
           <t>身体拘束の内容・目的・理由・拘束時間又は時間帯・期間・場所・改善に向けた取り組み方法を詳細に説明し、充分理解が得られるように努めます。</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="32" customHeight="1">
-      <c r="A83" s="5" t="inlineStr">
+    <row r="85" ht="32" customHeight="1">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t>また、身体拘束の同意期限を越え、なお拘束を必要とする場合については、事前に契約者・家族等と行っている内容と方向性、利用者の状態などを確認説明し、同意を得たうえで実施します。</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="6" customHeight="1"/>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="4" t="inlineStr">
+    <row r="86" ht="6" customHeight="1"/>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
         <is>
           <t>3）記録と再検討</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="64" customHeight="1">
-      <c r="A86" s="5" t="inlineStr">
+    <row r="88" ht="64" customHeight="1">
+      <c r="A88" s="5" t="inlineStr">
         <is>
           <t>法律上、身体拘束に関する記録は義務付けられており、専用の様式を用いてその態様及び時間・その際の利用者の心身の状況・やむを得なかった理由などを記録します。身体拘束の早期解除に向けて、拘束の必要性や方法を逐次検討します。その記録は5年間保存し、行政担当部局の運営指導等が行われる際に提示できるようにします。</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="6" customHeight="1"/>
-    <row r="88" ht="20" customHeight="1">
-      <c r="A88" s="4" t="inlineStr">
+    <row r="89" ht="6" customHeight="1"/>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>4）拘束の解除</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="32" customHeight="1">
-      <c r="A89" s="5" t="inlineStr">
+    <row r="91" ht="32" customHeight="1">
+      <c r="A91" s="5" t="inlineStr">
         <is>
           <t>3）の記録と再検討の結果、身体拘束を継続する必要性がなくなった場合は、速やかに身体拘束を解除します。その場合には、契約者、家族、居宅介護支援事業所に報告します。</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="10" customHeight="1"/>
-    <row r="91" ht="26" customHeight="1">
-      <c r="A91" s="16" t="inlineStr">
+    <row r="92" ht="10" customHeight="1"/>
+    <row r="93" ht="26" customHeight="1">
+      <c r="A93" s="16" t="inlineStr">
         <is>
           <t>5．身体的拘束等の報告方法等のための方策に関する基本方針</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="32" customHeight="1">
-      <c r="A92" s="5" t="inlineStr">
+    <row r="94" ht="32" customHeight="1">
+      <c r="A94" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">　1）身体的拘束等を行う場合には、4．の手続きに基づき利用者家族に速やかに説明し、報告を行うこと。</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="48" customHeight="1">
-      <c r="A93" s="5" t="inlineStr">
+    <row r="95" ht="48" customHeight="1">
+      <c r="A95" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">　2）訪問先等において他の職員等による適切な手続きに依らない身体的拘束等を視認等した場合、具体的な状況、時刻等を確認したうえで委員会への報告を行うこと。当該報告を受けた委員は、身体的拘束を実施したと思われる職員に聞き取りを行い実態の把握に努めること。</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="48" customHeight="1">
-      <c r="A94" s="5" t="inlineStr">
+    <row r="96" ht="48" customHeight="1">
+      <c r="A96" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">　3）適切な手続きに依らない身体的拘束の事実が判明した場合は、利用者及び利用者家族への謝罪を行い、大阪市への報告を行うこと。高齢者虐待に該当するおそれがある場合は、高齢者虐待防止法に基づき通報すること。</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="32" customHeight="1">
-      <c r="A95" s="5" t="inlineStr">
+    <row r="97" ht="32" customHeight="1">
+      <c r="A97" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">　4）訪問時に家族等による身体拘束を発見した場合は、管理者に報告し、居宅介護支援事業所と連携して対応すること。</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="8" customHeight="1"/>
-    <row r="97" ht="22" customHeight="1">
-      <c r="A97" s="17" t="inlineStr">
+    <row r="98" ht="8" customHeight="1"/>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="17" t="inlineStr">
         <is>
           <t>介護保険指定基準において身体拘束禁止の対象となる具体的な行為</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　（1）徘徊しないように、車椅子や椅子・ベッドに体幹や四肢をひも等で縛る</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="20" customHeight="1">
-      <c r="A99" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　（2）転落しないように、ベッドに体幹や四肢をひも等で縛る</t>
         </is>
       </c>
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　（3）自分で降りられないように、ベッドを柵（サイドレール）で囲む</t>
+          <t xml:space="preserve">　（1）徘徊しないように、車椅子や椅子・ベッドに体幹や四肢をひも等で縛る</t>
         </is>
       </c>
     </row>
     <row r="101" ht="20" customHeight="1">
       <c r="A101" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">　（2）転落しないように、ベッドに体幹や四肢をひも等で縛る</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（3）自分で降りられないように、ベッドを柵（サイドレール）で囲む</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">　（4）点滴・経管栄養等のチューブを抜かないように、四肢をひも等で縛る</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="32" customHeight="1">
-      <c r="A102" s="5" t="inlineStr">
+    <row r="104" ht="32" customHeight="1">
+      <c r="A104" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">　（5）点滴・経管栄養等のチューブを抜かないように、又は皮膚をかきむしらないように、手指の機能を制限するミトン型の手袋等をつける</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="32" customHeight="1">
-      <c r="A103" s="5" t="inlineStr">
+    <row r="105" ht="32" customHeight="1">
+      <c r="A105" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">　（6）車椅子・椅子からずり落ちたり、立ち上がったりしないように、Y字型拘束帯や腰ベルト・車椅子テーブルをつける</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="20" customHeight="1">
-      <c r="A104" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　（7）立ち上がる能力のある人の立ち上がりを妨げるような椅子を使用する</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="20" customHeight="1">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　（8）脱衣やオムツはずしを制限するために、介護衣（つなぎ服）を着せる</t>
         </is>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　（9）他人への迷惑行為を防ぐために、ベッドなどに体幹や四肢をひも等で縛る</t>
+          <t xml:space="preserve">　（7）立ち上がる能力のある人の立ち上がりを妨げるような椅子を使用する</t>
         </is>
       </c>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　（10）行動を落ち着かせるために、向精神薬を過剰に服用させる</t>
+          <t xml:space="preserve">　（8）脱衣やオムツはずしを制限するために、介護衣（つなぎ服）を着せる</t>
         </is>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">　（9）他人への迷惑行為を防ぐために、ベッドなどに体幹や四肢をひも等で縛る</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（10）行動を落ち着かせるために、向精神薬を過剰に服用させる</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">　（11）自分の意思で開けることのできない居室等に隔離する</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="8" customHeight="1"/>
-    <row r="110" ht="26" customHeight="1">
-      <c r="A110" s="16" t="inlineStr">
+    <row r="111" ht="8" customHeight="1"/>
+    <row r="112" ht="26" customHeight="1">
+      <c r="A112" s="16" t="inlineStr">
         <is>
           <t>6．身体拘束廃止に向けた各職種の役割</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="32" customHeight="1">
-      <c r="A111" s="5" t="inlineStr">
+    <row r="113" ht="32" customHeight="1">
+      <c r="A113" s="5" t="inlineStr">
         <is>
           <t>身体拘束の廃止のために、各職種の専門性に基づくアプローチから、チームケアを行うことを基本とし、それぞれの果たすべき役割に責任をもって対応します。</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="6" customHeight="1"/>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="4" t="inlineStr">
+    <row r="114" ht="6" customHeight="1"/>
+    <row r="115" ht="20" customHeight="1">
+      <c r="A115" s="4" t="inlineStr">
         <is>
           <t>（代表取締役）</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　1）身体拘束における諸課題等の最高責任者</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="20" customHeight="1">
-      <c r="A115" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　2）委員会総括責任者</t>
         </is>
       </c>
     </row>
     <row r="116" ht="20" customHeight="1">
       <c r="A116" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">　1）身体拘束における諸課題等の最高責任者</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="20" customHeight="1">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　2）委員会総括責任者</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="20" customHeight="1">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">　3）家族、医療、行政機関、その他関係機関への対応</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="8" customHeight="1"/>
-    <row r="118" ht="20" customHeight="1">
-      <c r="A118" s="4" t="inlineStr">
+    <row r="119" ht="8" customHeight="1"/>
+    <row r="120" ht="20" customHeight="1">
+      <c r="A120" s="4" t="inlineStr">
         <is>
           <t>（身体拘束適正化委員会）</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="20" customHeight="1">
-      <c r="A119" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　1）身体拘束廃止のための指針の周知徹底</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="20" customHeight="1">
-      <c r="A120" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　2）身体拘束に関する説明書、システムの確立</t>
         </is>
       </c>
     </row>
     <row r="121" ht="20" customHeight="1">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　3）身体拘束に関する対応策及び防止策の検討</t>
+          <t xml:space="preserve">　1）身体拘束廃止のための指針の周知徹底</t>
         </is>
       </c>
     </row>
     <row r="122" ht="20" customHeight="1">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　4）検討内容の実践、結果確認及び再検討</t>
+          <t xml:space="preserve">　2）身体拘束に関する説明書、システムの確立</t>
         </is>
       </c>
     </row>
     <row r="123" ht="20" customHeight="1">
       <c r="A123" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">　3）身体拘束に関する対応策及び防止策の検討</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="20" customHeight="1">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　4）検討内容の実践、結果確認及び再検討</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">　5）身体拘束廃止に向けた職員教育</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="8" customHeight="1"/>
-    <row r="125" ht="20" customHeight="1">
-      <c r="A125" s="4" t="inlineStr">
+    <row r="126" ht="8" customHeight="1"/>
+    <row r="127" ht="20" customHeight="1">
+      <c r="A127" s="4" t="inlineStr">
         <is>
           <t>（全従業者）</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="20" customHeight="1">
-      <c r="A126" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　1）拘束がもたらす弊害を正確に認識する</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="20" customHeight="1">
-      <c r="A127" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　2）利用者の尊厳を理解する</t>
         </is>
       </c>
     </row>
     <row r="128" ht="20" customHeight="1">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　3）利用者の疾病、障害等による行動特性の理解</t>
+          <t xml:space="preserve">　1）拘束がもたらす弊害を正確に認識する</t>
         </is>
       </c>
     </row>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　4）利用者個々の心身の状態を把握し、基本的ケアに努める</t>
+          <t xml:space="preserve">　2）利用者の尊厳を理解する</t>
         </is>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　5）利用者とのコミュニケーションを充分にとる</t>
+          <t xml:space="preserve">　3）利用者の疾病、障害等による行動特性の理解</t>
         </is>
       </c>
     </row>
     <row r="131" ht="20" customHeight="1">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　6）記録は正確かつ丁寧に記録する</t>
+          <t xml:space="preserve">　4）利用者個々の心身の状態を把握し、基本的ケアに努める</t>
         </is>
       </c>
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　7）医療機関、家族、居宅介護支援事業所等の関係機関との連絡調整</t>
+          <t xml:space="preserve">　5）利用者とのコミュニケーションを充分にとる</t>
         </is>
       </c>
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　8）訪問介護員が行える医療的ケアの範囲の確認</t>
+          <t xml:space="preserve">　6）記録は正確かつ丁寧に記録する</t>
         </is>
       </c>
     </row>
     <row r="134" ht="20" customHeight="1">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　9）重度化する利用者の状態観察</t>
+          <t xml:space="preserve">　7）医療機関、家族、居宅介護支援事業所等の関係機関との連絡調整</t>
         </is>
       </c>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　10）家族の意向に添ったケアの確立</t>
+          <t xml:space="preserve">　8）訪問介護員が行える医療的ケアの範囲の確認</t>
         </is>
       </c>
     </row>
     <row r="136" ht="20" customHeight="1">
       <c r="A136" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">　9）重度化する利用者の状態観察</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　10）家族の意向に添ったケアの確立</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="20" customHeight="1">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">　11）利用者宅の住環境（段差・家具配置等）や福祉用具の改善提案</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="8" customHeight="1"/>
-    <row r="138" ht="26" customHeight="1">
-      <c r="A138" s="16" t="inlineStr">
+    <row r="139" ht="8" customHeight="1"/>
+    <row r="140" ht="26" customHeight="1">
+      <c r="A140" s="16" t="inlineStr">
         <is>
           <t>7．身体拘束廃止・改善のための職員教育・研修</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="32" customHeight="1">
-      <c r="A139" s="5" t="inlineStr">
+    <row r="141" ht="32" customHeight="1">
+      <c r="A141" s="5" t="inlineStr">
         <is>
           <t>支援に携わる全ての職員（登録ヘルパーを含む）に対して、身体拘束廃止と人権を尊重したケアの励行を図り、事故防止と合わせてリスクマネジメントとしての職員教育を行います。</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="20" customHeight="1">
-      <c r="A140" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　① 定期的な教育・研修（年2回）の実施</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="20" customHeight="1">
-      <c r="A141" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　② 新任者に対する身体拘束廃止・改善のための研修の実施</t>
         </is>
       </c>
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">　① 定期的な教育・研修（年2回）の実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="20" customHeight="1">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　② 新任者に対する身体拘束廃止・改善のための研修の実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">　③ その他必要な教育・研修の実施</t>
         </is>
       </c>
     </row>
-    <row r="143" ht="8" customHeight="1"/>
-    <row r="144" ht="26" customHeight="1">
-      <c r="A144" s="16" t="inlineStr">
+    <row r="145" ht="8" customHeight="1"/>
+    <row r="146" ht="26" customHeight="1">
+      <c r="A146" s="16" t="inlineStr">
         <is>
           <t>8．身体拘束廃止に関する指針の閲覧について</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="32" customHeight="1">
-      <c r="A145" s="5" t="inlineStr">
+    <row r="147" ht="32" customHeight="1">
+      <c r="A147" s="5" t="inlineStr">
         <is>
           <t>この指針は、当事業所内に掲示するとともに、利用者・家族がいつでも自由に閲覧することができます。</t>
         </is>
       </c>
     </row>
-    <row r="146" ht="10" customHeight="1"/>
-    <row r="147" ht="26" customHeight="1">
-      <c r="A147" s="16" t="inlineStr">
+    <row r="148" ht="10" customHeight="1"/>
+    <row r="149" ht="26" customHeight="1">
+      <c r="A149" s="16" t="inlineStr">
         <is>
           <t>9．附則</t>
         </is>
       </c>
     </row>
-    <row r="148" ht="20" customHeight="1">
-      <c r="A148" s="5" t="inlineStr">
+    <row r="150" ht="20" customHeight="1">
+      <c r="A150" s="5" t="inlineStr">
         <is>
           <t>この指針は令和8年2月1日より施行する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="102">
+  <mergeCells count="104">
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="A142:E142"/>
     <mergeCell ref="A1:E1"/>
@@ -11561,15 +11587,15 @@
     <mergeCell ref="A94:E94"/>
     <mergeCell ref="A103:E103"/>
     <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A87:E87"/>
     <mergeCell ref="A128:E128"/>
+    <mergeCell ref="A137:E137"/>
     <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A89:E89"/>
     <mergeCell ref="A136:E136"/>
     <mergeCell ref="A105:E105"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A113:E113"/>
-    <mergeCell ref="A139:E139"/>
     <mergeCell ref="A71:E71"/>
     <mergeCell ref="A129:E129"/>
     <mergeCell ref="A91:E91"/>
@@ -11583,17 +11609,14 @@
     <mergeCell ref="A77:E77"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A83:E83"/>
-    <mergeCell ref="A148:E148"/>
     <mergeCell ref="A49:E49"/>
     <mergeCell ref="A138:E138"/>
     <mergeCell ref="A132:E132"/>
     <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A119:E119"/>
     <mergeCell ref="A69:E69"/>
-    <mergeCell ref="A78:E78"/>
     <mergeCell ref="A118:E118"/>
-    <mergeCell ref="A75:E75"/>
     <mergeCell ref="A133:E133"/>
+    <mergeCell ref="A80:E80"/>
     <mergeCell ref="A120:E120"/>
     <mergeCell ref="A95:E95"/>
     <mergeCell ref="A104:E104"/>
@@ -11603,59 +11626,64 @@
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A81:E81"/>
     <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A96:E96"/>
     <mergeCell ref="A147:E147"/>
     <mergeCell ref="A58:E58"/>
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="A67:E67"/>
-    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A73:E73"/>
     <mergeCell ref="A60:E60"/>
     <mergeCell ref="A123:E123"/>
     <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A146:E146"/>
+    <mergeCell ref="A124:E124"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A108:E108"/>
+    <mergeCell ref="A84:E84"/>
     <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A149:E149"/>
     <mergeCell ref="A50:E50"/>
-    <mergeCell ref="A86:E86"/>
     <mergeCell ref="A42:E42"/>
     <mergeCell ref="A141:E141"/>
     <mergeCell ref="A135:E135"/>
+    <mergeCell ref="A150:E150"/>
     <mergeCell ref="A144:E144"/>
     <mergeCell ref="A122:E122"/>
     <mergeCell ref="A125:E125"/>
-    <mergeCell ref="A72:E72"/>
     <mergeCell ref="A134:E134"/>
+    <mergeCell ref="A112:E112"/>
     <mergeCell ref="A121:E121"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A44:E44"/>
     <mergeCell ref="A127:E127"/>
     <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A114:E114"/>
     <mergeCell ref="A64:E64"/>
-    <mergeCell ref="A98:E98"/>
     <mergeCell ref="A51:E51"/>
     <mergeCell ref="A107:E107"/>
     <mergeCell ref="A61:E61"/>
     <mergeCell ref="A88:E88"/>
+    <mergeCell ref="A70:E70"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A90:E90"/>
     <mergeCell ref="A99:E99"/>
     <mergeCell ref="A74:E74"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A145:E145"/>
     <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A76:E76"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A85:E85"/>
     <mergeCell ref="A116:E116"/>
-    <mergeCell ref="A126:E126"/>
     <mergeCell ref="A140:E140"/>
     <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A109:E109"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A68:E68"/>
     <mergeCell ref="A102:E102"/>
-    <mergeCell ref="A111:E111"/>
-    <mergeCell ref="A92:E92"/>
+    <mergeCell ref="A117:E117"/>
+    <mergeCell ref="A143:E143"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11762,7 +11790,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>吉田 駿成</t>
+          <t>吉田 俊輔</t>
         </is>
       </c>
       <c r="C7" s="22" t="inlineStr">
@@ -11773,6 +11801,28 @@
       <c r="D7" s="22" t="inlineStr">
         <is>
           <t>身体拘束に関する諸課題の最高責任者、家族・医療・行政機関等への対応、指針の改廃の決定</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>委員</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>吉田 麻美</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>事務・総務</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>議事録の作成・保存、記録様式の管理、委員会資料の準備</t>
         </is>
       </c>
     </row>
@@ -11782,23 +11832,26 @@
           <t>【開催】年1回以上定期的に開催（感染症対策委員会・虐待防止委員会と同日に開催：6月・11月）。身体拘束の検討が必要なとき、適切な手続きによらない拘束が判明したとき等は随時開催する。</t>
         </is>
       </c>
+      <c r="B9" s="32" t="n"/>
+      <c r="C9" s="32" t="n"/>
+      <c r="D9" s="33" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t>【参加】必要に応じて、サービス提供責任者・当該利用者の担当訪問介護員・居宅介護支援事業所（ケアマネジャー）・主治医等の参加を求める。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="34" t="inlineStr">
         <is>
           <t>【記録】議事録を委員会ごとに作成し、全職員に周知のうえ5年間保存する。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="34" t="inlineStr">
         <is>
           <t>根拠：「身体拘束廃止に関する指針」3（1）</t>
         </is>
@@ -12599,7 +12652,7 @@
           <t>① 苦情・相談の受付</t>
         </is>
       </c>
-      <c r="C140" s="32" t="inlineStr">
+      <c r="C140" s="35" t="inlineStr">
         <is>
           <t>電話／対面／書面／代理で受理
 傾聴し、感情を受け止める
@@ -12620,7 +12673,7 @@
           <t>② 初期情報の記録</t>
         </is>
       </c>
-      <c r="C142" s="32" t="inlineStr">
+      <c r="C142" s="35" t="inlineStr">
         <is>
           <t>苦情（相談）記録表へ記入
 内容・緊急度・対象利用者を整理
@@ -12641,7 +12694,7 @@
           <t>③ 緊急度判定</t>
         </is>
       </c>
-      <c r="C144" s="32" t="inlineStr">
+      <c r="C144" s="35" t="inlineStr">
         <is>
           <t>【高】生命・安全に係る／重大クレーム
 【中】早急に対応が必要
@@ -12662,7 +12715,7 @@
           <t>④ 初期対応の実施</t>
         </is>
       </c>
-      <c r="C146" s="32" t="inlineStr">
+      <c r="C146" s="35" t="inlineStr">
         <is>
           <t>担当交代、訪問調整、緊急措置
 必要に応じて主治医・ケアマネへ連絡</t>
@@ -12682,7 +12735,7 @@
           <t>⑤ 事実確認</t>
         </is>
       </c>
-      <c r="C148" s="32" t="inlineStr">
+      <c r="C148" s="35" t="inlineStr">
         <is>
           <t>関係職員への聞き取り
 訪問記録・ケア記録との照合
@@ -12703,7 +12756,7 @@
           <t>⑥ 分析・判断</t>
         </is>
       </c>
-      <c r="C150" s="32" t="inlineStr">
+      <c r="C150" s="35" t="inlineStr">
         <is>
           <t>原因の特定（ヒューマンエラー／体制要因など）
 事業所としての判断と改善方針決定</t>
@@ -12723,7 +12776,7 @@
           <t>⑦ 利用者・家族への説明</t>
         </is>
       </c>
-      <c r="C152" s="32" t="inlineStr">
+      <c r="C152" s="35" t="inlineStr">
         <is>
           <t>事実確認結果と改善策を説明
 理解状況と同意の有無を記録</t>
@@ -12743,7 +12796,7 @@
           <t>⑧ 是正措置・改善策の実行</t>
         </is>
       </c>
-      <c r="C154" s="32" t="inlineStr">
+      <c r="C154" s="35" t="inlineStr">
         <is>
           <t>担当者変更／介助方法改善／研修の実施
 再発防止策を組織として実行</t>
@@ -12763,7 +12816,7 @@
           <t>⑨ フォローアップ</t>
         </is>
       </c>
-      <c r="C156" s="32" t="inlineStr">
+      <c r="C156" s="35" t="inlineStr">
         <is>
           <t>後日、利用者へ確認の連絡
 収束状況を記録、必要に応じて再対応</t>
@@ -12783,7 +12836,7 @@
           <t>⑩ 終結・保存</t>
         </is>
       </c>
-      <c r="C158" s="32" t="inlineStr">
+      <c r="C158" s="35" t="inlineStr">
         <is>
           <t>管理者が最終確認
 苦情（相談）記録表を保存（5年）
@@ -13786,7 +13839,7 @@
     <row r="11" ht="24" customHeight="1"/>
     <row r="12" ht="24" customHeight="1"/>
     <row r="13" ht="80" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>職場におけるハラスメントの
 防止に関する規定</t>
@@ -15023,7 +15076,7 @@
     <row r="11" ht="24" customHeight="1"/>
     <row r="12" ht="24" customHeight="1"/>
     <row r="13" ht="80" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>利用者等からのハラスメント
 防止・対応規程</t>
@@ -16027,7 +16080,7 @@
     <row r="11" ht="24" customHeight="1"/>
     <row r="12" ht="24" customHeight="1"/>
     <row r="13" ht="80" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>利用者等からのハラスメント
 防止・対応マニュアル</t>
@@ -18604,7 +18657,7 @@
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="34" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t>受付日</t>
         </is>
@@ -18615,7 +18668,7 @@
       <c r="E5" s="23" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="34" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>受付方法（電話・対面・書面・代理等）</t>
         </is>
@@ -18626,7 +18679,7 @@
       <c r="E6" s="23" t="n"/>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>苦情（相談）者氏名／続柄</t>
         </is>
@@ -18637,7 +18690,7 @@
       <c r="E7" s="23" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="34" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>対象利用者名</t>
         </is>
@@ -18648,7 +18701,7 @@
       <c r="E8" s="23" t="n"/>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="34" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>受付職員名</t>
         </is>
@@ -18659,7 +18712,7 @@
       <c r="E9" s="23" t="n"/>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="34" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>苦情（相談）区分
 （サービス内容・職員対応・安全衛生・事務手続・その他）</t>
@@ -18671,7 +18724,7 @@
       <c r="E10" s="23" t="n"/>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="34" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>発生日時・場所</t>
         </is>
@@ -18682,7 +18735,7 @@
       <c r="E11" s="23" t="n"/>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="34" t="inlineStr">
+      <c r="A12" s="37" t="inlineStr">
         <is>
           <t>緊急度（高・中・低）</t>
         </is>
@@ -18693,14 +18746,14 @@
       <c r="E12" s="23" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="35" t="inlineStr">
+      <c r="A14" s="38" t="inlineStr">
         <is>
           <t>1．苦情（相談）内容の詳細</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="36" t="inlineStr">
+      <c r="A15" s="39" t="inlineStr">
         <is>
           <t>（事実関係、発生状況、当事者の言動、経緯などを可能な限り具体的に記録）</t>
         </is>
@@ -18742,14 +18795,14 @@
       <c r="E20" s="23" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="35" t="inlineStr">
+      <c r="A22" s="38" t="inlineStr">
         <is>
           <t>2．利用者・家族の意向／感情の状況</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="36" t="inlineStr">
+      <c r="A23" s="39" t="inlineStr">
         <is>
           <t>（怒り・不安・困惑など、受け止め方を含めて明確に記述）</t>
         </is>
@@ -18777,14 +18830,14 @@
       <c r="E26" s="23" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="35" t="inlineStr">
+      <c r="A28" s="38" t="inlineStr">
         <is>
           <t>3．初期対応</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="36" t="inlineStr">
+      <c r="A29" s="39" t="inlineStr">
         <is>
           <t>（受付時の対応、説明内容、緊急対応の要否、関係者（管理者・ケアマネジャー・主治医等）への連絡など）</t>
         </is>
@@ -18812,14 +18865,14 @@
       <c r="E32" s="23" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="35" t="inlineStr">
+      <c r="A34" s="38" t="inlineStr">
         <is>
           <t>4．関係職員への聞き取り記録</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="36" t="inlineStr">
+      <c r="A35" s="39" t="inlineStr">
         <is>
           <t>（事実確認内容、職員の説明、第三者の証言等）</t>
         </is>
@@ -18854,14 +18907,14 @@
       <c r="E39" s="23" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="35" t="inlineStr">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>5．事業所としての分析・判断</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="36" t="inlineStr">
+      <c r="A42" s="39" t="inlineStr">
         <is>
           <t>（原因分析、再発要因、責任区分の検討など）</t>
         </is>
@@ -18889,14 +18942,14 @@
       <c r="E45" s="23" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="35" t="inlineStr">
+      <c r="A47" s="38" t="inlineStr">
         <is>
           <t>6．対応内容</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="36" t="inlineStr">
+      <c r="A48" s="39" t="inlineStr">
         <is>
           <t>（是正措置、改善策、訪問調整、担当変更、職員指導内容など）</t>
         </is>
@@ -18924,14 +18977,14 @@
       <c r="E51" s="23" t="n"/>
     </row>
     <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="35" t="inlineStr">
+      <c r="A53" s="38" t="inlineStr">
         <is>
           <t>7．利用者・家族への説明／同意</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="36" t="inlineStr">
+      <c r="A54" s="39" t="inlineStr">
         <is>
           <t>（説明日、説明者、理解状況、同意の有無）</t>
         </is>
@@ -18959,14 +19012,14 @@
       <c r="E57" s="23" t="n"/>
     </row>
     <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="35" t="inlineStr">
+      <c r="A59" s="38" t="inlineStr">
         <is>
           <t>8．再発防止策</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="36" t="inlineStr">
+      <c r="A60" s="39" t="inlineStr">
         <is>
           <t>（教育、マニュアル改訂、業務フロー改善等）</t>
         </is>
@@ -18994,14 +19047,14 @@
       <c r="E63" s="23" t="n"/>
     </row>
     <row r="65" ht="22" customHeight="1">
-      <c r="A65" s="35" t="inlineStr">
+      <c r="A65" s="38" t="inlineStr">
         <is>
           <t>9．フォローアップ記録</t>
         </is>
       </c>
     </row>
     <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="36" t="inlineStr">
+      <c r="A66" s="39" t="inlineStr">
         <is>
           <t>（後日の確認状況、苦情の収束状況、残課題、対応完了日など）</t>
         </is>
@@ -19029,14 +19082,14 @@
       <c r="E69" s="23" t="n"/>
     </row>
     <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="35" t="inlineStr">
+      <c r="A71" s="38" t="inlineStr">
         <is>
           <t>10．管理者コメント</t>
         </is>
       </c>
     </row>
     <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="36" t="inlineStr">
+      <c r="A72" s="39" t="inlineStr">
         <is>
           <t>（総括、必要な追加措置、大阪市・国保連への報告の要否、虐待・事故に該当する場合の通報・報告など）</t>
         </is>
@@ -19089,7 +19142,7 @@
       <c r="C79" s="9" t="n"/>
     </row>
     <row r="80" ht="20" customHeight="1">
-      <c r="A80" s="36" t="inlineStr">
+      <c r="A80" s="39" t="inlineStr">
         <is>
           <t>※本記録表は対応完了日から5年間保存する。</t>
         </is>

</xml_diff>

<commit_message>
議事録: replace facility wording, add 事業所名
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_社内規程一式.xlsx
+++ b/output/いいかいご_社内規程一式.xlsx
@@ -19387,7 +19387,7 @@
     <row r="3">
       <c r="B3" s="38" t="inlineStr">
         <is>
-          <t>（株式会社dhpケアマネジメント）</t>
+          <t>（株式会社dhpケアマネジメント　いいかいご）</t>
         </is>
       </c>
     </row>
@@ -19573,7 +19573,7 @@
       <c r="C25" s="46" t="inlineStr">
         <is>
           <t>・認知症進行による夜間不穏がある利用者について事例共有。
-・徘徊・転倒リスクに対し、環境整備や巡視頻度見直しなど拘束に頼らない予防策を検討。
+・徘徊・転倒リスクに対し、環境整備や、訪問時の見守り強化・訪問回数や時間帯の見直し（ケアマネジャーと相談）など拘束に頼らない予防策を検討。
 ・本人の生活リズム再評価、観察記録強化、家族との連携強化を決定。</t>
         </is>
       </c>

</xml_diff>

<commit_message>
研修報告書: visiting-care wording, title; align roster roles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_社内規程一式.xlsx
+++ b/output/いいかいご_社内規程一式.xlsx
@@ -8335,45 +8335,45 @@
       </c>
       <c r="D134" s="22" t="inlineStr">
         <is>
-          <t>感染症対策全体の統括・最終判断・行政報告。研修・教育担当を兼務</t>
+          <t>感染症対策全体の統括・最終判断・行政報告、研修講師・欠席者の補講</t>
         </is>
       </c>
       <c r="E134" s="23" t="n"/>
     </row>
-    <row r="135" ht="32" customHeight="1">
+    <row r="135" ht="48" customHeight="1">
       <c r="A135" s="20" t="inlineStr">
         <is>
-          <t>委員（代表取締役）</t>
+          <t>看護職委員</t>
         </is>
       </c>
       <c r="B135" s="21" t="n"/>
       <c r="C135" s="22" t="inlineStr">
         <is>
-          <t>吉田 俊輔</t>
+          <t>松村 知恵</t>
         </is>
       </c>
       <c r="D135" s="22" t="inlineStr">
         <is>
-          <t>法人としての方針決定、BCPの承認、重大事案時の対外対応</t>
+          <t>トリアージ・医療的助言・PPE指導、BCPレベル判断の承認（委員長と2名承認）</t>
         </is>
       </c>
       <c r="E135" s="23" t="n"/>
     </row>
-    <row r="136" ht="48" customHeight="1">
+    <row r="136" ht="32" customHeight="1">
       <c r="A136" s="20" t="inlineStr">
         <is>
-          <t>看護職委員</t>
+          <t>委員（代表取締役）</t>
         </is>
       </c>
       <c r="B136" s="21" t="n"/>
       <c r="C136" s="22" t="inlineStr">
         <is>
-          <t>松村 知恵</t>
+          <t>吉田 俊輔</t>
         </is>
       </c>
       <c r="D136" s="22" t="inlineStr">
         <is>
-          <t>医療的助言・トリアージ・PPE指導、BCPレベル判断の承認（委員長と2名承認）</t>
+          <t>感染疑い時の訪問調整（担当者限定・訪問順の変更）、BCPの承認</t>
         </is>
       </c>
       <c r="E136" s="23" t="n"/>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="D137" s="22" t="inlineStr">
         <is>
-          <t>議事録作成、記録整備・行政書類確認、衛生用品の在庫管理</t>
+          <t>行政報告ルートの確認、議事録・記録整備、衛生用品の在庫管理</t>
         </is>
       </c>
       <c r="E137" s="23" t="n"/>
@@ -8400,7 +8400,7 @@
     <row r="138" ht="32" customHeight="1">
       <c r="A138" s="20" t="inlineStr">
         <is>
-          <t>委員（ヘルパー代表）</t>
+          <t>委員（研修・教育担当）</t>
         </is>
       </c>
       <c r="B138" s="21" t="n"/>
@@ -8411,7 +8411,7 @@
       </c>
       <c r="D138" s="22" t="inlineStr">
         <is>
-          <t>現場情報共有・フィードバック、標準予防策の実施状況の確認</t>
+          <t>研修の体系化、欠席者へのフォロー、現場情報の共有</t>
         </is>
       </c>
       <c r="E138" s="23" t="n"/>
@@ -19417,14 +19417,14 @@
     <row r="2">
       <c r="B2" s="37" t="inlineStr">
         <is>
-          <t>株式会社dhpケアマネジメント</t>
+          <t>株式会社dhpケアマネジメント　いいかいご</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="38" t="inlineStr">
         <is>
-          <t>感染症対策委員会 研修実施報告書（統合版）</t>
+          <t>感染症対策委員会 研修・訓練実施報告書（統合版）</t>
         </is>
       </c>
     </row>
@@ -19432,14 +19432,14 @@
     <row r="5" ht="24" customHeight="1">
       <c r="B5" s="39" t="inlineStr">
         <is>
-          <t>1．研修実施報告書</t>
+          <t>1．研修・訓練実施報告書</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="B6" s="40" t="inlineStr">
         <is>
-          <t>■ 研修日時</t>
+          <t>■ 研修・訓練日時</t>
         </is>
       </c>
       <c r="C6" s="41" t="inlineStr">
@@ -19452,7 +19452,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="B7" s="40" t="inlineStr">
         <is>
-          <t>■ 研修内容</t>
+          <t>■ 研修・訓練内容</t>
         </is>
       </c>
       <c r="C7" s="41" t="inlineStr">
@@ -19465,7 +19465,7 @@
     <row r="8" ht="26" customHeight="1">
       <c r="B8" s="40" t="inlineStr">
         <is>
-          <t>■ 研修場所</t>
+          <t>■ 実施場所</t>
         </is>
       </c>
       <c r="C8" s="41" t="inlineStr">
@@ -19492,7 +19492,7 @@
     <row r="10" ht="44" customHeight="1">
       <c r="B10" s="40" t="inlineStr">
         <is>
-          <t>■ 研修参加者</t>
+          <t>■ 参加者</t>
         </is>
       </c>
       <c r="C10" s="41" t="inlineStr">
@@ -19529,8 +19529,8 @@
       </c>
       <c r="C12" s="41" t="inlineStr">
         <is>
-          <t>今回の夏季感染対策研修では、委員会メンバー全員が一丸となり、初動対応・ゾーンニング・BCP運用の要点を明確に整理できたことが大きな成果でした。特に、想定訓練において動線遮断やPPE装着といった具体的オペレーションを確認したことにより、実際の発生時に迷いが生じにくい体制が構築できています。
-課題として浮き彫りになったPPE配置の分かりづらさや、判断基準の統一については、委員として責任を持って改善し、現場にとってより安全で実務的な仕組みへ進化させていきます。今後も“早期把握・早期遮断・正確な対応”を軸に、利用者とスタッフ双方の安全を守り抜く体制づくりを進めていきます。</t>
+          <t>今回の夏季感染対策研修では、委員会メンバー全員が一丸となり、初動対応・感染疑い時の訪問調整・BCP運用の要点を明確に整理できたことが大きな成果でした。特に、想定訓練において感染疑い利用者宅への訪問調整（担当者限定・訪問順の変更）やPPE装着といった具体的オペレーションを確認したことにより、実際の発生時に迷いが生じにくい体制が構築できています。
+課題として浮き彫りになった訪問用衛生用品セットの内容・在庫の分かりづらさや、判断基準の統一については、委員として責任を持って改善し、現場にとってより安全で実務的な仕組みへ進化させていきます。今後も“早期把握・早期遮断・正確な対応”を軸に、利用者とスタッフ双方の安全を守り抜く体制づくりを進めていきます。</t>
         </is>
       </c>
       <c r="D12" s="42" t="n"/>
@@ -19605,7 +19605,7 @@
         <is>
           <t>・生田：統括
 ・松村：トリアージ・医療的助言
-・吉田（俊）：導線遮断・ゾーニング
+・吉田（俊）：感染疑い時の訪問調整（担当者限定・訪問順の変更）
 ・吉田（麻）：行政報告ルート確認
 ・win yadanar aung：研修体系化と欠席フォロー</t>
         </is>
@@ -19637,8 +19637,8 @@
       <c r="C21" s="41" t="inlineStr">
         <is>
           <t>・グローブ二重装着
-・ガウン着脱の注意点
-・廃棄物処理とゾーニング</t>
+・ガウン着脱の注意点（利用者宅の玄関等での着脱手順）
+・使用済みPPE・廃棄物の密閉処理（利用者宅のごみ出しルールに従う）</t>
         </is>
       </c>
       <c r="D21" s="42" t="n"/>
@@ -19651,8 +19651,8 @@
       </c>
       <c r="C22" s="41" t="inlineStr">
         <is>
-          <t>・温度管理
-・搬入物検品
+          <t>・調理援助時の温度管理
+・購入食品・冷蔵庫内食品の消費期限確認
 ・嘔吐物処理手順</t>
         </is>
       </c>
@@ -19666,7 +19666,7 @@
       </c>
       <c r="C23" s="41" t="inlineStr">
         <is>
-          <t>・巡回チェック表簡素化
+          <t>・訪問時の体調確認チェック表の簡素化
 ・月次ミニ研修
 ・行政書類テンプレ改善</t>
         </is>
@@ -19689,8 +19689,8 @@
       </c>
       <c r="C26" s="41" t="inlineStr">
         <is>
-          <t>・導線遮断に3分の遅れ
-・PPE在庫の把握に差
+          <t>・感染疑い時の訪問調整（担当者限定・訪問順の変更）の判断に3分の遅れ
+・訪問用PPE・衛生用品の在庫把握に差
 ・嘔吐物処理セットの補充漏れ
 ・BCPレベル判断の迷い</t>
         </is>
@@ -19705,8 +19705,8 @@
       </c>
       <c r="C27" s="41" t="inlineStr">
         <is>
-          <t>・初動カードを電話横へ配置
-・PPE棚の色分け・写真表示
+          <t>・初動カードを事業所の電話横へ配置し、訪問用バッグにも携行
+・訪問用衛生用品セットの中身を写真付きで一覧表示
 ・嘔吐物処理セットの月2回点検
 ・BCP基準は生田・松村の2名承認制</t>
         </is>
@@ -19737,7 +19737,7 @@
     <row r="31" ht="24" customHeight="1">
       <c r="B31" s="45" t="inlineStr">
         <is>
-          <t>5. 訓練実施責任者</t>
+          <t>5. 研修・訓練実施責任者</t>
         </is>
       </c>
       <c r="C31" s="46" t="inlineStr">
@@ -19750,7 +19750,7 @@
     <row r="32" ht="24" customHeight="1">
       <c r="B32" s="45" t="inlineStr">
         <is>
-          <t>6. 訓練記録作成者</t>
+          <t>6. 研修・訓練記録作成者</t>
         </is>
       </c>
       <c r="C32" s="46" t="inlineStr">

</xml_diff>

<commit_message>
Unify spelling: WIN YADANAR AUNG
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_社内規程一式.xlsx
+++ b/output/いいかいご_社内規程一式.xlsx
@@ -8406,7 +8406,7 @@
       <c r="B138" s="21" t="n"/>
       <c r="C138" s="22" t="inlineStr">
         <is>
-          <t>WIN YADANAR AWNG</t>
+          <t>WIN YADANAR AUNG</t>
         </is>
       </c>
       <c r="D138" s="22" t="inlineStr">
@@ -11248,7 +11248,7 @@
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　・訪問介護員（ヘルパー代表）　WIN YADANAR AWNG</t>
+          <t xml:space="preserve">　・訪問介護員（ヘルパー代表）　WIN YADANAR AUNG</t>
         </is>
       </c>
     </row>
@@ -12001,7 +12001,7 @@
       </c>
       <c r="B10" s="22" t="inlineStr">
         <is>
-          <t>WIN YADANAR AWNG</t>
+          <t>WIN YADANAR AUNG</t>
         </is>
       </c>
       <c r="C10" s="22" t="inlineStr">
@@ -19498,7 +19498,7 @@
       <c r="C10" s="41" t="inlineStr">
         <is>
           <t>委員長：生田友哉
-委員：松村知恵、win yadanar aung、吉田俊輔、吉田麻美</t>
+委員：松村知恵、WIN YADANAR AUNG、吉田俊輔、吉田麻美</t>
         </is>
       </c>
       <c r="D10" s="42" t="n"/>
@@ -19607,7 +19607,7 @@
 ・松村：トリアージ・医療的助言
 ・吉田（俊）：感染疑い時の訪問調整（担当者限定・訪問順の変更）
 ・吉田（麻）：行政報告ルート確認
-・win yadanar aung：研修体系化と欠席フォロー</t>
+・WIN YADANAR AUNG：研修体系化と欠席フォロー</t>
         </is>
       </c>
       <c r="D19" s="42" t="n"/>
@@ -19896,7 +19896,7 @@
       </c>
       <c r="C13" s="46" t="inlineStr">
         <is>
-          <t>松村知恵、win yadanar aung、吉田俊輔、吉田麻美</t>
+          <t>松村知恵、WIN YADANAR AUNG、吉田俊輔、吉田麻美</t>
         </is>
       </c>
       <c r="D13" s="42" t="n"/>
@@ -20099,7 +20099,7 @@
     <row r="36" ht="28" customHeight="1">
       <c r="B36" s="51" t="inlineStr">
         <is>
-          <t>win yadanar aung（委員）</t>
+          <t>WIN YADANAR AUNG（委員）</t>
         </is>
       </c>
       <c r="C36" s="52" t="inlineStr">

</xml_diff>

<commit_message>
Unify representative name to 吉田駿成
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_社内規程一式.xlsx
+++ b/output/いいかいご_社内規程一式.xlsx
@@ -8369,7 +8369,7 @@
       <c r="B136" s="21" t="n"/>
       <c r="C136" s="22" t="inlineStr">
         <is>
-          <t>吉田 俊輔</t>
+          <t>吉田 駿成</t>
         </is>
       </c>
       <c r="D136" s="22" t="inlineStr">
@@ -11228,7 +11228,7 @@
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">　・代表取締役（法人代表者）　吉田 俊輔</t>
+          <t xml:space="preserve">　・代表取締役（法人代表者）　吉田 駿成</t>
         </is>
       </c>
     </row>
@@ -11936,7 +11936,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>吉田 俊輔</t>
+          <t>吉田 駿成</t>
         </is>
       </c>
       <c r="C7" s="22" t="inlineStr">
@@ -19499,7 +19499,7 @@
       <c r="C10" s="41" t="inlineStr">
         <is>
           <t>委員長：生田友哉
-委員：松村知恵、WIN YADANAR AUNG、吉田俊輔、吉田麻美</t>
+委員：松村知恵、WIN YADANAR AUNG、吉田駿成、吉田麻美</t>
         </is>
       </c>
       <c r="D10" s="42" t="n"/>
@@ -19606,7 +19606,7 @@
         <is>
           <t>・生田：統括
 ・松村：トリアージ・医療的助言
-・吉田（俊）：感染疑い時の訪問調整（担当者限定・訪問順の変更）
+・吉田（駿）：感染疑い時の訪問調整（担当者限定・訪問順の変更）
 ・吉田（麻）：行政報告ルート確認
 ・WIN YADANAR AUNG：研修体系化と欠席フォロー</t>
         </is>
@@ -19897,7 +19897,7 @@
       </c>
       <c r="C13" s="46" t="inlineStr">
         <is>
-          <t>松村知恵、WIN YADANAR AUNG、吉田俊輔、吉田麻美</t>
+          <t>松村知恵、WIN YADANAR AUNG、吉田駿成、吉田麻美</t>
         </is>
       </c>
       <c r="D13" s="42" t="n"/>
@@ -20113,7 +20113,7 @@
     <row r="37" ht="28" customHeight="1">
       <c r="B37" s="51" t="inlineStr">
         <is>
-          <t>吉田俊輔（委員）</t>
+          <t>吉田駿成（委員）</t>
         </is>
       </c>
       <c r="C37" s="52" t="inlineStr">
@@ -20278,7 +20278,7 @@
       <c r="C10" s="41" t="inlineStr">
         <is>
           <t>委員長：生田友哉
-委員：WIN YADANAR AUNG、吉田俊輔、吉田麻美</t>
+委員：WIN YADANAR AUNG、吉田駿成、吉田麻美</t>
         </is>
       </c>
       <c r="D10" s="42" t="n"/>

</xml_diff>

<commit_message>
Add PDF versions of all documents and a zip bundle
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_社内規程一式.xlsx
+++ b/output/いいかいご_社内規程一式.xlsx
@@ -19792,6 +19792,7 @@
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -20170,6 +20171,7 @@
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -20497,6 +20499,7 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -20679,6 +20682,7 @@
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C8:D8"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>